<commit_message>
Add MEAE international-student TL;DR sheet (exclude Work-Study and undergrad-only)
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -10,10 +10,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="岗位检索" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整中文" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="英文原文" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MEAE国际学生省流版" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'岗位检索'!$A$4:$W$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'MEAE国际学生省流版'!$A$4:$G$93</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33419,6 +33421,3144 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G93"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MEAE 国际学生省流版</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>面向 MEAE 硕士国际学生（F-1）· 已排除 33 个必须勤工助学或仅限本科的岗位 · 快照 2026-08-16T05:02:08.919027+08:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="6" customHeight="1"/>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>职位</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>部门</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>每周工时</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>时薪</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>截止日期</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>注意</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>学生质量保证实习生</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>大学信息技术部·校级支持服务</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>学生 IT 支持技术员</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>犹他自然历史博物馆</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>$17</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>研究生研究助理（NoTB）</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>社会工作学院</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>未提供</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>需社工硕士/博士在读，会 Mplus/SPSS/R</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>人体艺术模特</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>艺术与艺术史系</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>0-6</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>$20</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>博物馆展品支架制作师（临时）</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>犹他自然历史博物馆</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>$35</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>需驾照；需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>兼职社交媒体内容助理</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>KUER 公共广播电台</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>$17</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>活动执勤警员</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>公共安全部·特别活动</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>$57.75</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>需驾照；需犹他州 LEO 认证+在职执法人员、美国公民/合法永久居民</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>卖场助理</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>校园商店</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>19-20</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>DOE</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>幼儿教师</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>学生家长支持中心</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>$15.5</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>食品证可后考；需经验；需 CPR/急救证，能抱举幼儿</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>校内托育课堂助理</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>学生家长支持中心</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>up to 19 hours/week, depending on hiring needs and incumbent schedule</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>$14.5</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>食品证可后考；入职 60 天内需食品证、TB 检测、BCI 背景调查、急救培训</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>考试服务技术员</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>在线教育</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>$12</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>收发货班次负责人</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>校园商店</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>$16</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>韩语兼职讲师</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>世界语言与文化系</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>4,200-6,000</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>需驾照；韩语接近母语级</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>市场内容实习生</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>校友关系办公室</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>8-10</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>校友社交媒体实习生</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>校友关系办公室</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>活动工作人员</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>校友关系办公室</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>15-19</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>$15.6</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Research Quest 市场营销实习生</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>犹他自然历史博物馆</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>需经验；需本科学历+2年经验 或 硕士</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>课程助教／教学助理</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>高管教育</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>15 to 19</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>楼宇服务助理</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Marriott 图书馆运营</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>能提举 25 磅、爬梯凳</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>古生物藏品与登记助理</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>犹他自然历史博物馆</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>$15.6</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>需经验；需通过背景调查</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>场馆餐饮区域协调员</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Rice-Eccles 体育场</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>16 hours per week or less</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>$18</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>设施维护助理</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>体育部</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>$16</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>需驾照；需经验；能提举 60 磅、需美国驾照</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Bennion Center 学生摄影师</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Bennion 社区参与中心</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>As needed</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>成人教育项目助理</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Red Butte 植物园</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>$16</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>需驾照；需经验；能提举 50 磅、走崎岖地形</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>现场服务办公室助理</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>S.J. Quinney 法学院</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>$9.62</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>学生网络布线技术员</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>信息管理</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>15 - 19</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Prosperity U 活动实习生</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>商业、健康与繁荣中心</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>$12</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Adobe 创意软件顾问</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>大学信息技术部·数字学习技术</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>需精通至少 4 款 Adobe 应用</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>学生媒体办公室副经理</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>学生媒体委员会</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>15-20</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>$11</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>办公室助理</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>犹他纳米制造实验室</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>$7.25</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>青少年项目助理</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>犹他自然历史博物馆</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>需驾照；需经验；需本科学历、驾照</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>酒店前台文员</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>大学宾馆</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>公众项目助理</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>犹他自然历史博物馆</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>学生参与项目视频实习生</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>校友关系办公室</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>15-19</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>需会视频剪辑（Pr/达芬奇等）、DSLR/微单</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>兼职临时学位进度审核专员</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>教务注册办公室</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>$20</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>需经验；需本科学历 + 1 年相关经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>停车管理巡查员</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>通勤服务</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>$18</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>需驾照；需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>学业导师</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>体育部</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>$11</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>需经验；需通过 BCI 背景调查</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>活动商品与运营助理</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>校园商店</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>$18</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>需驾照</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>招生办公室学生文员</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>招生办公室</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>15-19 hours weekly</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>$14</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>学生住宿大使</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>住宿与居住教育</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>19.99</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>$14</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>Prosperity U 社交媒体实习生</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>商业、健康与繁荣中心</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>$14</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>建筑与规划学院学生大使</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>建筑与规划学院</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>8-12</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>活动支持专员</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Red Butte 植物园</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>$15.5</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>办公室与课堂支持助理</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>高管教育</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>10–19 hours per week, with the potential for increased hours during the summer.</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>国际学生与学者服务同伴助理</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>国际学生与学者服务中心</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>学生系统管理员（二级）</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Marriott 图书馆运营</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>$16</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>需熟悉 Jamf Pro / SCCM，会脚本（Bash/PowerShell/Python/C/C++）</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>数据治理传播实习生</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>大学分析与机构报告</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>19 hours</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>数据治理技术实习生</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>大学分析与机构报告</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>19 hours per week</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>酒店夜班前台文员</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>大学宾馆</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>$19</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>兼职保洁员</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>住宿与居住教育</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>$16.16</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>临时啤酒售卖员</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Rice-Eccles 体育场</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>$19</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>年满 21 岁、需酒类服务证</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>SCIF 可持续发展大使</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>可持续校园倡议基金</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>$16</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>实践学习可持续发展大使</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>可持续校园倡议基金</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>$16</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>电子与计算机工程系行政助理</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>电子与计算机工程系</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>$7.25</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>场馆餐饮技术支持专员</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>Rice-Eccles 体育场</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>$16</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>社交媒体实习生</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>多学科设计系</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="n">
+        <v>57</v>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>STEMCAP 项目助理</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>本科生教育倡导项目</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>$25</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="n">
+        <v>58</v>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>舞台经理</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>音乐学院</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>Varries based on performance/event schedule</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>$13</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>需经验；需 2 年剧场舞台技术经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>MHA 职业服务经理兼职业教练</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>高管教育</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>$30</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>市场营销助理</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>学生会</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>up to 19 hours/week</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>$14</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>Utech 技术服务助理</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>校园商店</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>19-20</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>需通过安全审查（security clearance）</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="n">
+        <v>62</v>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>订单履约助理</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>校园商店</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>$14.5</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="n">
+        <v>63</v>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>校内体育裁判（勤工助学）</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>校内体育</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>$12</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>需 CPR 认证（可入职一月内取得）</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="n">
+        <v>64</v>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>仓库工作人员</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Rice-Eccles 体育场</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>4 hours per week or less</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>$16</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>体育场餐饮售卖人员</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>Rice-Eccles 体育场</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>需食品证</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="n">
+        <v>66</v>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>兼职保洁员</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>住宿与居住教育</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>$16.16</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>UMFA 咖啡馆后厨工作人员</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>犹他美术博物馆</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>1-19</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>$14</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>需食品证</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>UMFA 商店店员</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>犹他美术博物馆</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>1-19</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>$13.65</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="n">
+        <v>69</v>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>夜班安保车司机</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>通勤服务</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>15-19 hours per week</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>$15.38</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>需驾照</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>顾客服务代表</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>财务与运营</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>$16</t>
+        </is>
+      </c>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="n">
+        <v>71</v>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>数据录入专员</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>高管教育</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>15-19</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>UMFA 活动工作人员</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>犹他美术博物馆</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>0-19</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>$13.65</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>需经验；能提举 50 磅</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="n">
+        <v>73</v>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>校园班车司机</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>通勤服务</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>$20</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>需 CDL 驾照（提供付费培训）</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="n">
+        <v>74</v>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>兼职保洁员</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>住宿与居住教育</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>$16.16</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>市场营销助理</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>校园健康中心</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>$14.5</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="n">
+        <v>76</v>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>教材与课程资料助理</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>校园商店</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>19-20</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>$14.5</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="G80" s="5" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="n">
+        <v>77</v>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>UMFA 安保服务人员</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>犹他美术博物馆</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>1-19</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>$13.65</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr">
+        <is>
+          <t>需驾照；需经验；需通过背景调查</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="n">
+        <v>78</v>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>Wilkes 中心学生大使</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>Wilkes 气候科学与政策中心</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>$14</t>
+        </is>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>社会工作学院兼职讲师</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>社会工作学院</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>20000 to 500000</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>实验室助理</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Huntsman 癌症研究所·Chandrasekharan 实验室</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>$7.25</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="G84" s="5" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="n">
+        <v>81</v>
+      </c>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>前厅收银员</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>先锋剧院</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>15-20</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>$11</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="B86" s="6" t="inlineStr">
+        <is>
+          <t>票房售票员</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>先锋剧院</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="inlineStr">
+        <is>
+          <t>$10.5</t>
+        </is>
+      </c>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="n">
+        <v>83</v>
+      </c>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>行政文员</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>校园卡服务</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>15-19 hours per week</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="G87" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="n">
+        <v>84</v>
+      </c>
+      <c r="B88" s="6" t="inlineStr">
+        <is>
+          <t>舞台技术员</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>UtahPresents 演出项目</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="inlineStr">
+        <is>
+          <t>$16</t>
+        </is>
+      </c>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="B89" s="6" t="inlineStr">
+        <is>
+          <t>网球中心前台工作人员</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>体育部</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E89" s="4" t="inlineStr">
+        <is>
+          <t>$7.25</t>
+        </is>
+      </c>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="G89" s="5" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="n">
+        <v>86</v>
+      </c>
+      <c r="B90" s="6" t="inlineStr">
+        <is>
+          <t>UCL 兼职讲师</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>英语语言学院</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="inlineStr">
+        <is>
+          <t>$49</t>
+        </is>
+      </c>
+      <c r="F90" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-13</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr">
+        <is>
+          <t>需 TESOL 硕士 + TESOL 证书</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="n">
+        <v>87</v>
+      </c>
+      <c r="B91" s="6" t="inlineStr">
+        <is>
+          <t>住宿招生与外联协调员</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>影响力与繁荣中心</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>15-19</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="inlineStr">
+        <is>
+          <t>$12</t>
+        </is>
+      </c>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="n">
+        <v>88</v>
+      </c>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>舞蹈学院摄像人员</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>舞蹈学院</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E92" s="4" t="inlineStr">
+        <is>
+          <t>$13.5</t>
+        </is>
+      </c>
+      <c r="F92" s="4" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="n">
+        <v>89</v>
+      </c>
+      <c r="B93" s="6" t="inlineStr">
+        <is>
+          <t>舞蹈学院舞台工作人员</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>舞蹈学院</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>$13.5</t>
+        </is>
+      </c>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:G93"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B43" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B50" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B51" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B52" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B53" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B54" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B56" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B57" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B58" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B59" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B60" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B61" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B62" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B63" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B64" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B65" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B66" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B67" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B68" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B69" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B70" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B71" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B72" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B73" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B74" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B75" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B76" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B77" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B78" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B79" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B80" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B81" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B82" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B83" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B84" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B85" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B86" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B87" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B88" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B89" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B90" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B91" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B92" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B93" r:id="rId89"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Exclude citizenship-required and closed jobs from intl sheet; document screening criteria
- add requires_citizenship detection (US citizen/national/LPR -> hard blocker for F-1)
- MEAE intl sheet now excludes Work-Study required, undergrad-only, closed, citizenship-required
- document screening criteria in README for future re-analysis
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'岗位检索'!$A$4:$W$126</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'MEAE国际学生省流版'!$A$4:$G$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'MEAE国际学生省流版'!$A$4:$G$90</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33421,7 +33421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G93"/>
+  <dimension ref="A1:G90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -33443,7 +33443,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>面向 MEAE 硕士国际学生（F-1）· 已排除 33 个必须勤工助学或仅限本科的岗位 · 快照 2026-08-16T05:02:08.919027+08:00</t>
+          <t>面向 MEAE 硕士国际学生（F-1）· 已排除 36 个必须勤工助学、仅限本科、已关闭或需公民身份的岗位 · 快照 2026-08-16T05:02:08.919027+08:00</t>
         </is>
       </c>
     </row>
@@ -33693,34 +33693,30 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>活动执勤警员</t>
+          <t>卖场助理</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>公共安全部·特别活动</t>
+          <t>校园商店</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>19-20</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>$57.75</t>
+          <t>DOE</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>需驾照；需犹他州 LEO 认证+在职执法人员、美国公民/合法永久居民</t>
-        </is>
-      </c>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -33728,30 +33724,34 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>卖场助理</t>
+          <t>幼儿教师</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>校园商店</t>
+          <t>学生家长支持中心</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>19-20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>DOE</t>
+          <t>$15.5</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr"/>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>食品证可后考；需经验；需 CPR/急救证，能抱举幼儿</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -33759,7 +33759,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>幼儿教师</t>
+          <t>校内托育课堂助理</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -33769,12 +33769,12 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>up to 19 hours/week, depending on hiring needs and incumbent schedule</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>$15.5</t>
+          <t>$14.5</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -33784,7 +33784,7 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>食品证可后考；需经验；需 CPR/急救证，能抱举幼儿</t>
+          <t>食品证可后考；入职 60 天内需食品证、TB 检测、BCI 背景调查、急救培训</t>
         </is>
       </c>
     </row>
@@ -33794,34 +33794,30 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>校内托育课堂助理</t>
+          <t>考试服务技术员</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>学生家长支持中心</t>
+          <t>在线教育</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>up to 19 hours/week, depending on hiring needs and incumbent schedule</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>$14.5</t>
+          <t>$12</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>食品证可后考；入职 60 天内需食品证、TB 检测、BCI 背景调查、急救培训</t>
-        </is>
-      </c>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -33829,22 +33825,22 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>考试服务技术员</t>
+          <t>收发货班次负责人</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>在线教育</t>
+          <t>校园商店</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>$12</t>
+          <t>$16</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -33852,7 +33848,11 @@
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr"/>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
@@ -33860,12 +33860,12 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>收发货班次负责人</t>
+          <t>韩语兼职讲师</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>校园商店</t>
+          <t>世界语言与文化系</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -33875,17 +33875,17 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>$16</t>
+          <t>4,200-6,000</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>需经验</t>
+          <t>需驾照；韩语接近母语级</t>
         </is>
       </c>
     </row>
@@ -33895,22 +33895,22 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>韩语兼职讲师</t>
+          <t>市场内容实习生</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>世界语言与文化系</t>
+          <t>校友关系办公室</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>8-10</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>4,200-6,000</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -33918,11 +33918,7 @@
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>需驾照；韩语接近母语级</t>
-        </is>
-      </c>
+      <c r="G17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
@@ -33930,7 +33926,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>市场内容实习生</t>
+          <t>校友社交媒体实习生</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -33940,7 +33936,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>8-10</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -33961,7 +33957,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>校友社交媒体实习生</t>
+          <t>活动工作人员</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -33971,12 +33967,12 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>15-19</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$15.6</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -33992,22 +33988,22 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>活动工作人员</t>
+          <t>Research Quest 市场营销实习生</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>校友关系办公室</t>
+          <t>犹他自然历史博物馆</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>15-19</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>$15.6</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -34015,7 +34011,11 @@
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>需经验；需本科学历+2年经验 或 硕士</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
@@ -34023,17 +34023,17 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Research Quest 市场营销实习生</t>
+          <t>课程助教／教学助理</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>犹他自然历史博物馆</t>
+          <t>高管教育</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15 to 19</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -34048,7 +34048,7 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>需经验；需本科学历+2年经验 或 硕士</t>
+          <t>需经验</t>
         </is>
       </c>
     </row>
@@ -34058,17 +34058,17 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>课程助教／教学助理</t>
+          <t>楼宇服务助理</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>高管教育</t>
+          <t>Marriott 图书馆运营</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>15 to 19</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -34078,12 +34078,12 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>需经验</t>
+          <t>能提举 25 磅、爬梯凳</t>
         </is>
       </c>
     </row>
@@ -34093,32 +34093,32 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>楼宇服务助理</t>
+          <t>古生物藏品与登记助理</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Marriott 图书馆运营</t>
+          <t>犹他自然历史博物馆</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$15.6</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>能提举 25 磅、爬梯凳</t>
+          <t>需经验；需通过背景调查</t>
         </is>
       </c>
     </row>
@@ -34128,32 +34128,32 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>古生物藏品与登记助理</t>
+          <t>场馆餐饮区域协调员</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>犹他自然历史博物馆</t>
+          <t>Rice-Eccles 体育场</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>16 hours per week or less</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>$15.6</t>
+          <t>$18</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>需经验；需通过背景调查</t>
+          <t>需经验</t>
         </is>
       </c>
     </row>
@@ -34163,32 +34163,32 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>场馆餐饮区域协调员</t>
+          <t>设施维护助理</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Rice-Eccles 体育场</t>
+          <t>体育部</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>16 hours per week or less</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>$18</t>
+          <t>$16</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>需经验</t>
+          <t>需驾照；需经验；能提举 60 磅、需美国驾照</t>
         </is>
       </c>
     </row>
@@ -34198,34 +34198,30 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>设施维护助理</t>
+          <t>Bennion Center 学生摄影师</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>体育部</t>
+          <t>Bennion 社区参与中心</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>As needed</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>$16</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>需驾照；需经验；能提举 60 磅、需美国驾照</t>
-        </is>
-      </c>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -34233,22 +34229,22 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Bennion Center 学生摄影师</t>
+          <t>成人教育项目助理</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Bennion 社区参与中心</t>
+          <t>Red Butte 植物园</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>As needed</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$16</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -34256,7 +34252,11 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr"/>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>需驾照；需经验；能提举 50 磅、走崎岖地形</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
@@ -34264,12 +34264,12 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>成人教育项目助理</t>
+          <t>现场服务办公室助理</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Red Butte 植物园</t>
+          <t>S.J. Quinney 法学院</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -34279,7 +34279,7 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>$16</t>
+          <t>$9.62</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -34289,7 +34289,7 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>需驾照；需经验；能提举 50 磅、走崎岖地形</t>
+          <t>需经验</t>
         </is>
       </c>
     </row>
@@ -34299,22 +34299,22 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>现场服务办公室助理</t>
+          <t>学生网络布线技术员</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>S.J. Quinney 法学院</t>
+          <t>信息管理</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>15 - 19</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>$9.62</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -34322,11 +34322,7 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr">
-        <is>
-          <t>需经验</t>
-        </is>
-      </c>
+      <c r="G29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
@@ -34334,22 +34330,22 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>学生网络布线技术员</t>
+          <t>Prosperity U 活动实习生</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>信息管理</t>
+          <t>商业、健康与繁荣中心</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>15 - 19</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$12</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -34365,22 +34361,22 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Prosperity U 活动实习生</t>
+          <t>Adobe 创意软件顾问</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>商业、健康与繁荣中心</t>
+          <t>大学信息技术部·数字学习技术</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>$12</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -34388,7 +34384,11 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr"/>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>需精通至少 4 款 Adobe 应用</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
@@ -34396,22 +34396,22 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Adobe 创意软件顾问</t>
+          <t>学生媒体办公室副经理</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>大学信息技术部·数字学习技术</t>
+          <t>学生媒体委员会</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>15-20</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$11</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -34419,11 +34419,7 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="G32" s="5" t="inlineStr">
-        <is>
-          <t>需精通至少 4 款 Adobe 应用</t>
-        </is>
-      </c>
+      <c r="G32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -34431,22 +34427,22 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>学生媒体办公室副经理</t>
+          <t>办公室助理</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>学生媒体委员会</t>
+          <t>犹他纳米制造实验室</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>15-20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>$11</t>
+          <t>$7.25</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -34462,12 +34458,12 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>办公室助理</t>
+          <t>青少年项目助理</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>犹他纳米制造实验室</t>
+          <t>犹他自然历史博物馆</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -34477,15 +34473,19 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>$7.25</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="G34" s="5" t="inlineStr"/>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>需驾照；需经验；需本科学历、驾照</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
@@ -34493,12 +34493,12 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>青少年项目助理</t>
+          <t>酒店前台文员</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>犹他自然历史博物馆</t>
+          <t>大学宾馆</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -34513,12 +34513,12 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>需驾照；需经验；需本科学历、驾照</t>
+          <t>需经验</t>
         </is>
       </c>
     </row>
@@ -34528,12 +34528,12 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>酒店前台文员</t>
+          <t>公众项目助理</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>大学宾馆</t>
+          <t>犹他自然历史博物馆</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -34563,17 +34563,17 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>公众项目助理</t>
+          <t>学生参与项目视频实习生</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>犹他自然历史博物馆</t>
+          <t>校友关系办公室</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>15-19</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
@@ -34583,12 +34583,12 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>需经验</t>
+          <t>需会视频剪辑（Pr/达芬奇等）、DSLR/微单</t>
         </is>
       </c>
     </row>
@@ -34598,32 +34598,32 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>学生参与项目视频实习生</t>
+          <t>兼职临时学位进度审核专员</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>校友关系办公室</t>
+          <t>教务注册办公室</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>15-19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$20</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>需会视频剪辑（Pr/达芬奇等）、DSLR/微单</t>
+          <t>需经验；需本科学历 + 1 年相关经验</t>
         </is>
       </c>
     </row>
@@ -34633,32 +34633,32 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>兼职临时学位进度审核专员</t>
+          <t>停车管理巡查员</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>教务注册办公室</t>
+          <t>通勤服务</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>$20</t>
+          <t>$18</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>需经验；需本科学历 + 1 年相关经验</t>
+          <t>需驾照；需经验</t>
         </is>
       </c>
     </row>
@@ -34668,12 +34668,12 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>停车管理巡查员</t>
+          <t>学业导师</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>通勤服务</t>
+          <t>体育部</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -34683,17 +34683,17 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>$18</t>
+          <t>$11</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>需驾照；需经验</t>
+          <t>需经验；需通过 BCI 背景调查</t>
         </is>
       </c>
     </row>
@@ -34703,22 +34703,22 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>学业导师</t>
+          <t>活动商品与运营助理</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>体育部</t>
+          <t>校园商店</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>$11</t>
+          <t>$18</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
@@ -34728,7 +34728,7 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>需经验；需通过 BCI 背景调查</t>
+          <t>需驾照</t>
         </is>
       </c>
     </row>
@@ -34738,34 +34738,30 @@
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>活动商品与运营助理</t>
+          <t>招生办公室学生文员</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>校园商店</t>
+          <t>招生办公室</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>15-19 hours weekly</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>$18</t>
+          <t>$14</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="inlineStr">
-        <is>
-          <t>需驾照</t>
-        </is>
-      </c>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
@@ -34773,17 +34769,17 @@
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>招生办公室学生文员</t>
+          <t>学生住宿大使</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>招生办公室</t>
+          <t>住宿与居住教育</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>15-19 hours weekly</t>
+          <t>19.99</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
@@ -34793,7 +34789,7 @@
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr"/>
@@ -34804,17 +34800,17 @@
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>学生住宿大使</t>
+          <t>Prosperity U 社交媒体实习生</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>住宿与居住教育</t>
+          <t>商业、健康与繁荣中心</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>19.99</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
@@ -34835,22 +34831,22 @@
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>Prosperity U 社交媒体实习生</t>
+          <t>建筑与规划学院学生大使</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>商业、健康与繁荣中心</t>
+          <t>建筑与规划学院</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>8-12</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>$14</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
@@ -34866,30 +34862,34 @@
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>建筑与规划学院学生大使</t>
+          <t>活动支持专员</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>建筑与规划学院</t>
+          <t>Red Butte 植物园</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>8-12</t>
+          <t>29</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$15.5</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="G46" s="5" t="inlineStr"/>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -34897,22 +34897,22 @@
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>活动支持专员</t>
+          <t>办公室与课堂支持助理</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Red Butte 植物园</t>
+          <t>高管教育</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>10–19 hours per week, with the potential for increased hours during the summer.</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>$15.5</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -34920,11 +34920,7 @@
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="G47" s="5" t="inlineStr">
-        <is>
-          <t>需经验</t>
-        </is>
-      </c>
+      <c r="G47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n">
@@ -34932,17 +34928,17 @@
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>办公室与课堂支持助理</t>
+          <t>国际学生与学者服务同伴助理</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>高管教育</t>
+          <t>国际学生与学者服务中心</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>10–19 hours per week, with the potential for increased hours during the summer.</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
@@ -34952,7 +34948,7 @@
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr"/>
@@ -34963,30 +34959,34 @@
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>国际学生与学者服务同伴助理</t>
+          <t>学生系统管理员（二级）</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>国际学生与学者服务中心</t>
+          <t>Marriott 图书馆运营</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$16</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="G49" s="5" t="inlineStr"/>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>需熟悉 Jamf Pro / SCCM，会脚本（Bash/PowerShell/Python/C/C++）</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="n">
@@ -34994,34 +34994,30 @@
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>学生系统管理员（二级）</t>
+          <t>数据治理传播实习生</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Marriott 图书馆运营</t>
+          <t>大学分析与机构报告</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>19 hours</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>$16</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="G50" s="5" t="inlineStr">
-        <is>
-          <t>需熟悉 Jamf Pro / SCCM，会脚本（Bash/PowerShell/Python/C/C++）</t>
-        </is>
-      </c>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
@@ -35029,7 +35025,7 @@
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>数据治理传播实习生</t>
+          <t>数据治理技术实习生</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
@@ -35039,7 +35035,7 @@
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>19 hours</t>
+          <t>19 hours per week</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
@@ -35060,22 +35056,22 @@
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>数据治理技术实习生</t>
+          <t>酒店夜班前台文员</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>大学分析与机构报告</t>
+          <t>大学宾馆</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>19 hours per week</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$19</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
@@ -35083,7 +35079,11 @@
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="G52" s="5" t="inlineStr"/>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
@@ -35091,34 +35091,30 @@
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>酒店夜班前台文员</t>
+          <t>兼职保洁员</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>大学宾馆</t>
+          <t>住宿与居住教育</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>$19</t>
+          <t>$16.16</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="G53" s="5" t="inlineStr">
-        <is>
-          <t>需经验</t>
-        </is>
-      </c>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n">
@@ -35126,30 +35122,34 @@
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>兼职保洁员</t>
+          <t>临时啤酒售卖员</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>住宿与居住教育</t>
+          <t>Rice-Eccles 体育场</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>10-15</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>$16.16</t>
+          <t>$19</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="G54" s="5" t="inlineStr"/>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>年满 21 岁、需酒类服务证</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="n">
@@ -35157,22 +35157,22 @@
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>临时啤酒售卖员</t>
+          <t>SCIF 可持续发展大使</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Rice-Eccles 体育场</t>
+          <t>可持续校园倡议基金</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>$19</t>
+          <t>$16</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
@@ -35180,11 +35180,7 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="G55" s="5" t="inlineStr">
-        <is>
-          <t>年满 21 岁、需酒类服务证</t>
-        </is>
-      </c>
+      <c r="G55" s="5" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="n">
@@ -35192,7 +35188,7 @@
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>SCIF 可持续发展大使</t>
+          <t>实践学习可持续发展大使</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
@@ -35223,22 +35219,22 @@
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>实践学习可持续发展大使</t>
+          <t>电子与计算机工程系行政助理</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>可持续校园倡议基金</t>
+          <t>电子与计算机工程系</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>$16</t>
+          <t>$7.25</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
@@ -35254,30 +35250,34 @@
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>电子与计算机工程系行政助理</t>
+          <t>场馆餐饮技术支持专员</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>电子与计算机工程系</t>
+          <t>Rice-Eccles 体育场</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>$7.25</t>
+          <t>$16</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="G58" s="5" t="inlineStr"/>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="n">
@@ -35285,12 +35285,12 @@
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>场馆餐饮技术支持专员</t>
+          <t>社交媒体实习生</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Rice-Eccles 体育场</t>
+          <t>多学科设计系</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -35300,7 +35300,7 @@
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>$16</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
@@ -35308,11 +35308,7 @@
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="G59" s="5" t="inlineStr">
-        <is>
-          <t>需经验</t>
-        </is>
-      </c>
+      <c r="G59" s="5" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="n">
@@ -35320,22 +35316,22 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>社交媒体实习生</t>
+          <t>STEMCAP 项目助理</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>多学科设计系</t>
+          <t>本科生教育倡导项目</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$25</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
@@ -35343,7 +35339,11 @@
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="G60" s="5" t="inlineStr"/>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="n">
@@ -35351,22 +35351,22 @@
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>STEMCAP 项目助理</t>
+          <t>舞台经理</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>本科生教育倡导项目</t>
+          <t>音乐学院</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>Varries based on performance/event schedule</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>$25</t>
+          <t>$13</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
@@ -35376,7 +35376,7 @@
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>需经验</t>
+          <t>需经验；需 2 年剧场舞台技术经验</t>
         </is>
       </c>
     </row>
@@ -35386,22 +35386,22 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>舞台经理</t>
+          <t>MHA 职业服务经理兼职业教练</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>音乐学院</t>
+          <t>高管教育</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>Varries based on performance/event schedule</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>$13</t>
+          <t>$30</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
@@ -35411,7 +35411,7 @@
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>需经验；需 2 年剧场舞台技术经验</t>
+          <t>需经验</t>
         </is>
       </c>
     </row>
@@ -35421,34 +35421,30 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>MHA 职业服务经理兼职业教练</t>
+          <t>市场营销助理</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>高管教育</t>
+          <t>学生会</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>up to 19 hours/week</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>$30</t>
+          <t>$14</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="G63" s="5" t="inlineStr">
-        <is>
-          <t>需经验</t>
-        </is>
-      </c>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="4" t="n">
@@ -35456,30 +35452,34 @@
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>市场营销助理</t>
+          <t>Utech 技术服务助理</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>学生会</t>
+          <t>校园商店</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>up to 19 hours/week</t>
+          <t>19-20</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>$14</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="G64" s="5" t="inlineStr"/>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>需通过安全审查（security clearance）</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="n">
@@ -35487,7 +35487,7 @@
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>Utech 技术服务助理</t>
+          <t>订单履约助理</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
@@ -35497,24 +35497,20 @@
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>19-20</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$14.5</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="G65" s="5" t="inlineStr">
-        <is>
-          <t>需通过安全审查（security clearance）</t>
-        </is>
-      </c>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="n">
@@ -35522,30 +35518,34 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>订单履约助理</t>
+          <t>校内体育裁判（勤工助学）</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>校园商店</t>
+          <t>校内体育</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>$14.5</t>
+          <t>$12</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="G66" s="5" t="inlineStr"/>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>需 CPR 认证（可入职一月内取得）</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="n">
@@ -35553,32 +35553,32 @@
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>校内体育裁判（勤工助学）</t>
+          <t>仓库工作人员</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>校内体育</t>
+          <t>Rice-Eccles 体育场</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>4 hours per week or less</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>$12</t>
+          <t>$16</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>需 CPR 认证（可入职一月内取得）</t>
+          <t>需经验</t>
         </is>
       </c>
     </row>
@@ -35588,7 +35588,7 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>仓库工作人员</t>
+          <t>体育场餐饮售卖人员</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
@@ -35598,12 +35598,12 @@
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>4 hours per week or less</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>$16</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr">
@@ -35613,7 +35613,7 @@
       </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
-          <t>需经验</t>
+          <t>需食品证</t>
         </is>
       </c>
     </row>
@@ -35623,22 +35623,22 @@
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>体育场餐饮售卖人员</t>
+          <t>兼职保洁员</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Rice-Eccles 体育场</t>
+          <t>住宿与居住教育</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$16.16</t>
         </is>
       </c>
       <c r="F69" s="4" t="inlineStr">
@@ -35646,11 +35646,7 @@
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="G69" s="5" t="inlineStr">
-        <is>
-          <t>需食品证</t>
-        </is>
-      </c>
+      <c r="G69" s="5" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="4" t="n">
@@ -35658,22 +35654,22 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>兼职保洁员</t>
+          <t>UMFA 咖啡馆后厨工作人员</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>住宿与居住教育</t>
+          <t>犹他美术博物馆</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>1-19</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>$16.16</t>
+          <t>$14</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr">
@@ -35681,7 +35677,11 @@
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="G70" s="5" t="inlineStr"/>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>需食品证</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="n">
@@ -35689,7 +35689,7 @@
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>UMFA 咖啡馆后厨工作人员</t>
+          <t>UMFA 商店店员</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
@@ -35704,7 +35704,7 @@
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>$14</t>
+          <t>$13.65</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr">
@@ -35714,7 +35714,7 @@
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>需食品证</t>
+          <t>需经验</t>
         </is>
       </c>
     </row>
@@ -35724,32 +35724,32 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>UMFA 商店店员</t>
+          <t>夜班安保车司机</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>犹他美术博物馆</t>
+          <t>通勤服务</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>1-19</t>
+          <t>15-19 hours per week</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>$13.65</t>
+          <t>$15.38</t>
         </is>
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>需经验</t>
+          <t>需驾照</t>
         </is>
       </c>
     </row>
@@ -35759,32 +35759,32 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>夜班安保车司机</t>
+          <t>顾客服务代表</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>通勤服务</t>
+          <t>财务与运营</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>15-19 hours per week</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>$15.38</t>
+          <t>$16</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>需驾照</t>
+          <t>需经验</t>
         </is>
       </c>
     </row>
@@ -35794,32 +35794,32 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>顾客服务代表</t>
+          <t>UMFA 活动工作人员</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>财务与运营</t>
+          <t>犹他美术博物馆</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>0-19</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>$16</t>
+          <t>$13.65</t>
         </is>
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>需经验</t>
+          <t>需经验；能提举 50 磅</t>
         </is>
       </c>
     </row>
@@ -35829,32 +35829,32 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>数据录入专员</t>
+          <t>校园班车司机</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>高管教育</t>
+          <t>通勤服务</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>15-19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$20</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>已关闭</t>
+          <t>需 CDL 驾照（提供付费培训）</t>
         </is>
       </c>
     </row>
@@ -35864,34 +35864,30 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>UMFA 活动工作人员</t>
+          <t>兼职保洁员</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>犹他美术博物馆</t>
+          <t>住宿与居住教育</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>0-19</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>$13.65</t>
+          <t>$16.16</t>
         </is>
       </c>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="G76" s="5" t="inlineStr">
-        <is>
-          <t>需经验；能提举 50 磅</t>
-        </is>
-      </c>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="n">
@@ -35899,34 +35895,30 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>校园班车司机</t>
+          <t>市场营销助理</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>通勤服务</t>
+          <t>校园健康中心</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>$20</t>
+          <t>$14.5</t>
         </is>
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="G77" s="5" t="inlineStr">
-        <is>
-          <t>需 CDL 驾照（提供付费培训）</t>
-        </is>
-      </c>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="n">
@@ -35934,27 +35926,27 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>兼职保洁员</t>
+          <t>教材与课程资料助理</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>住宿与居住教育</t>
+          <t>校园商店</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>19-20</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>$16.16</t>
+          <t>$14.5</t>
         </is>
       </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr"/>
@@ -35965,30 +35957,34 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>市场营销助理</t>
+          <t>UMFA 安保服务人员</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>校园健康中心</t>
+          <t>犹他美术博物馆</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>1-19</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>$14.5</t>
+          <t>$13.65</t>
         </is>
       </c>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="G79" s="5" t="inlineStr"/>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>需驾照；需经验；需通过背景调查</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="n">
@@ -35996,27 +35992,27 @@
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>教材与课程资料助理</t>
+          <t>Wilkes 中心学生大使</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>校园商店</t>
+          <t>Wilkes 气候科学与政策中心</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>19-20</t>
+          <t>10-15</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>$14.5</t>
+          <t>$14</t>
         </is>
       </c>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="G80" s="5" t="inlineStr"/>
@@ -36027,34 +36023,30 @@
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>UMFA 安保服务人员</t>
+          <t>实验室助理</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>犹他美术博物馆</t>
+          <t>Huntsman 癌症研究所·Chandrasekharan 实验室</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>1-19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>$13.65</t>
+          <t>$7.25</t>
         </is>
       </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="G81" s="5" t="inlineStr">
-        <is>
-          <t>需驾照；需经验；需通过背景调查</t>
-        </is>
-      </c>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="n">
@@ -36062,30 +36054,34 @@
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>Wilkes 中心学生大使</t>
+          <t>前厅收银员</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>Wilkes 气候科学与政策中心</t>
+          <t>先锋剧院</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>15-20</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>$14</t>
+          <t>$11</t>
         </is>
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
-        </is>
-      </c>
-      <c r="G82" s="5" t="inlineStr"/>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="n">
@@ -36093,32 +36089,32 @@
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>社会工作学院兼职讲师</t>
+          <t>票房售票员</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>社会工作学院</t>
+          <t>先锋剧院</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>20000 to 500000</t>
+          <t>$10.5</t>
         </is>
       </c>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-11-03</t>
         </is>
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>已关闭</t>
+          <t>需经验</t>
         </is>
       </c>
     </row>
@@ -36128,22 +36124,22 @@
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>实验室助理</t>
+          <t>行政文员</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>Huntsman 癌症研究所·Chandrasekharan 实验室</t>
+          <t>校园卡服务</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>15-19 hours per week</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>$7.25</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="F84" s="4" t="inlineStr">
@@ -36151,7 +36147,11 @@
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="G84" s="5" t="inlineStr"/>
+      <c r="G84" s="5" t="inlineStr">
+        <is>
+          <t>需经验</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n">
@@ -36159,27 +36159,27 @@
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>前厅收银员</t>
+          <t>舞台技术员</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>先锋剧院</t>
+          <t>UtahPresents 演出项目</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>15-20</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t>$11</t>
+          <t>$16</t>
         </is>
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>2026-11-03</t>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">
@@ -36194,34 +36194,30 @@
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>票房售票员</t>
+          <t>网球中心前台工作人员</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>先锋剧院</t>
+          <t>体育部</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>$10.5</t>
+          <t>$7.25</t>
         </is>
       </c>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>2026-11-03</t>
-        </is>
-      </c>
-      <c r="G86" s="5" t="inlineStr">
-        <is>
-          <t>需经验</t>
-        </is>
-      </c>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="n">
@@ -36229,32 +36225,32 @@
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>行政文员</t>
+          <t>UCL 兼职讲师</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>校园卡服务</t>
+          <t>英语语言学院</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>15-19 hours per week</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$49</t>
         </is>
       </c>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>2026-11-03</t>
+          <t>2026-11-13</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>需经验</t>
+          <t>需 TESOL 硕士 + TESOL 证书</t>
         </is>
       </c>
     </row>
@@ -36264,34 +36260,30 @@
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>舞台技术员</t>
+          <t>住宿招生与外联协调员</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>UtahPresents 演出项目</t>
+          <t>影响力与繁荣中心</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15-19</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>$16</t>
+          <t>$12</t>
         </is>
       </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>2026-11-05</t>
-        </is>
-      </c>
-      <c r="G88" s="5" t="inlineStr">
-        <is>
-          <t>需经验</t>
-        </is>
-      </c>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="n">
@@ -36299,27 +36291,27 @@
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>网球中心前台工作人员</t>
+          <t>舞蹈学院摄像人员</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>体育部</t>
+          <t>舞蹈学院</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>$7.25</t>
+          <t>$13.5</t>
         </is>
       </c>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>2026-11-07</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr"/>
@@ -36330,130 +36322,33 @@
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>UCL 兼职讲师</t>
+          <t>舞蹈学院舞台工作人员</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>英语语言学院</t>
+          <t>舞蹈学院</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>$49</t>
+          <t>$13.5</t>
         </is>
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>2026-11-13</t>
-        </is>
-      </c>
-      <c r="G90" s="5" t="inlineStr">
-        <is>
-          <t>需 TESOL 硕士 + TESOL 证书</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="4" t="n">
-        <v>87</v>
-      </c>
-      <c r="B91" s="6" t="inlineStr">
-        <is>
-          <t>住宿招生与外联协调员</t>
-        </is>
-      </c>
-      <c r="C91" s="5" t="inlineStr">
-        <is>
-          <t>影响力与繁荣中心</t>
-        </is>
-      </c>
-      <c r="D91" s="4" t="inlineStr">
-        <is>
-          <t>15-19</t>
-        </is>
-      </c>
-      <c r="E91" s="4" t="inlineStr">
-        <is>
-          <t>$12</t>
-        </is>
-      </c>
-      <c r="F91" s="4" t="inlineStr">
-        <is>
-          <t>2026-11-20</t>
-        </is>
-      </c>
-      <c r="G91" s="5" t="inlineStr"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="4" t="n">
-        <v>88</v>
-      </c>
-      <c r="B92" s="6" t="inlineStr">
-        <is>
-          <t>舞蹈学院摄像人员</t>
-        </is>
-      </c>
-      <c r="C92" s="5" t="inlineStr">
-        <is>
-          <t>舞蹈学院</t>
-        </is>
-      </c>
-      <c r="D92" s="4" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E92" s="4" t="inlineStr">
-        <is>
-          <t>$13.5</t>
-        </is>
-      </c>
-      <c r="F92" s="4" t="inlineStr">
-        <is>
           <t>2026-12-31</t>
         </is>
       </c>
-      <c r="G92" s="5" t="inlineStr"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="4" t="n">
-        <v>89</v>
-      </c>
-      <c r="B93" s="6" t="inlineStr">
-        <is>
-          <t>舞蹈学院舞台工作人员</t>
-        </is>
-      </c>
-      <c r="C93" s="5" t="inlineStr">
-        <is>
-          <t>舞蹈学院</t>
-        </is>
-      </c>
-      <c r="D93" s="4" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E93" s="4" t="inlineStr">
-        <is>
-          <t>$13.5</t>
-        </is>
-      </c>
-      <c r="F93" s="4" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
-      </c>
-      <c r="G93" s="5" t="inlineStr"/>
+      <c r="G90" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G93"/>
+  <autoFilter ref="A4:G90"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
@@ -36545,9 +36440,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B88" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B89" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B90" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B91" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B92" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B93" r:id="rId89"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add core-skills field, beautify README with badges and TOC
- add data/core-skills.json (core abilities: photography, editing, design, programming...)
- surface 核心能力 column in MEAE intl sheet
- README: shields.io badges, table of contents, fix stale 酒类证 mention
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'岗位检索'!$A$4:$W$126</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'MEAE国际学生省流版'!$A$4:$G$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'MEAE国际学生省流版'!$A$4:$H$90</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33421,16 +33421,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G90"/>
+  <dimension ref="A1:H90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -33461,25 +33462,30 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
+          <t>核心能力</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
           <t>部门</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>每周工时</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>时薪</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>截止日期</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>注意</t>
         </is>
@@ -33496,25 +33502,30 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
+          <t>软件测试</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
           <t>大学信息技术部·校级支持服务</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -33527,25 +33538,30 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
+          <t>IT 技术支持</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
           <t>犹他自然历史博物馆</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>$17</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -33562,25 +33578,30 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
+          <t>统计分析、研究</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
           <t>社会工作学院</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>未提供</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>需社工硕士/博士在读，会 Mplus/SPSS/R</t>
         </is>
@@ -33597,25 +33618,30 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
+          <t>人体模特</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
           <t>艺术与艺术史系</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>0-6</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>$20</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr"/>
+      <c r="H8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -33628,25 +33654,30 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
+          <t>展品制作、手工</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
           <t>犹他自然历史博物馆</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>10-15</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>$35</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>需驾照；需经验</t>
         </is>
@@ -33663,25 +33694,30 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
+          <t>社交媒体运营</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
           <t>KUER 公共广播电台</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>$17</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -33696,27 +33732,28 @@
           <t>卖场助理</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr"/>
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>校园商店</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>19-20</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>DOE</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr"/>
+      <c r="H11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -33729,25 +33766,30 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
+          <t>幼儿教育</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
           <t>学生家长支持中心</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>$15.5</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>食品证可后考；需经验；需 CPR/急救证，能抱举幼儿</t>
         </is>
@@ -33764,25 +33806,30 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
+          <t>幼教辅助</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
           <t>学生家长支持中心</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>up to 19 hours/week, depending on hiring needs and incumbent schedule</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>$14.5</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>食品证可后考；入职 60 天内需食品证、TB 检测、BCI 背景调查、急救培训</t>
         </is>
@@ -33799,25 +33846,30 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
+          <t>考试服务、技术支持</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
           <t>在线教育</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>$12</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr"/>
+      <c r="H14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -33828,27 +33880,28 @@
           <t>收发货班次负责人</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr"/>
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>校园商店</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>$16</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -33865,25 +33918,30 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
+          <t>韩语教学</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
           <t>世界语言与文化系</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>4,200-6,000</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>需驾照；韩语接近母语级</t>
         </is>
@@ -33900,25 +33958,30 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
+          <t>内容创作、营销</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
           <t>校友关系办公室</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>8-10</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr"/>
+      <c r="H17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
@@ -33931,25 +33994,30 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
+          <t>社交媒体运营</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
           <t>校友关系办公室</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr"/>
+      <c r="H18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -33960,27 +34028,28 @@
           <t>活动工作人员</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr"/>
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>校友关系办公室</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>15-19</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>$15.6</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr"/>
+      <c r="H19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
@@ -33993,25 +34062,30 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
+          <t>市场调研</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
           <t>犹他自然历史博物馆</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>需经验；需本科学历+2年经验 或 硕士</t>
         </is>
@@ -34028,25 +34102,30 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
+          <t>教学辅助</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
           <t>高管教育</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>15 to 19</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="H21" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -34061,27 +34140,28 @@
           <t>楼宇服务助理</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr"/>
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>Marriott 图书馆运营</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>能提举 25 磅、爬梯凳</t>
         </is>
@@ -34096,27 +34176,28 @@
           <t>古生物藏品与登记助理</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr"/>
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>犹他自然历史博物馆</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>$15.6</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>需经验；需通过背景调查</t>
         </is>
@@ -34133,25 +34214,30 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
+          <t>餐饮协调</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
           <t>Rice-Eccles 体育场</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>16 hours per week or less</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>$18</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -34166,27 +34252,28 @@
           <t>设施维护助理</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr"/>
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>体育部</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>$16</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>需驾照；需经验；能提举 60 磅、需美国驾照</t>
         </is>
@@ -34203,25 +34290,30 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
+          <t>摄影</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
           <t>Bennion 社区参与中心</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>As needed</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr"/>
+      <c r="H26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -34232,27 +34324,28 @@
           <t>成人教育项目助理</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr"/>
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>Red Butte 植物园</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>$16</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
+      <c r="H27" s="5" t="inlineStr">
         <is>
           <t>需驾照；需经验；能提举 50 磅、走崎岖地形</t>
         </is>
@@ -34267,27 +34360,28 @@
           <t>现场服务办公室助理</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr"/>
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>S.J. Quinney 法学院</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>$9.62</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -34304,25 +34398,30 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
+          <t>网络布线</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
           <t>信息管理</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>15 - 19</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr"/>
+      <c r="H29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
@@ -34335,25 +34434,30 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
+          <t>活动策划</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
           <t>商业、健康与繁荣中心</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t>$12</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr"/>
+      <c r="H30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -34366,25 +34470,30 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
+          <t>Adobe 设计</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
           <t>大学信息技术部·数字学习技术</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="H31" s="5" t="inlineStr">
         <is>
           <t>需精通至少 4 款 Adobe 应用</t>
         </is>
@@ -34401,25 +34510,30 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
+          <t>媒体运营</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
           <t>学生媒体委员会</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
         <is>
           <t>15-20</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>$11</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="G32" s="4" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="G32" s="5" t="inlineStr"/>
+      <c r="H32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -34430,27 +34544,28 @@
           <t>办公室助理</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr"/>
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>犹他纳米制造实验室</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="F33" s="4" t="inlineStr">
         <is>
           <t>$7.25</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="G33" s="4" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr"/>
+      <c r="H33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
@@ -34463,25 +34578,30 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
+          <t>青少年项目</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
           <t>犹他自然历史博物馆</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="G34" s="4" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="G34" s="5" t="inlineStr">
+      <c r="H34" s="5" t="inlineStr">
         <is>
           <t>需驾照；需经验；需本科学历、驾照</t>
         </is>
@@ -34496,27 +34616,28 @@
           <t>酒店前台文员</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr"/>
+      <c r="D35" s="5" t="inlineStr">
         <is>
           <t>大学宾馆</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="G35" s="4" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="G35" s="5" t="inlineStr">
+      <c r="H35" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -34533,25 +34654,30 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
+          <t>公众项目、教育</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
           <t>犹他自然历史博物馆</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="E36" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="F36" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
+      <c r="G36" s="4" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="G36" s="5" t="inlineStr">
+      <c r="H36" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -34568,25 +34694,30 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
+          <t>视频拍摄剪辑</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
           <t>校友关系办公室</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="E37" s="4" t="inlineStr">
         <is>
           <t>15-19</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="F37" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr">
+      <c r="G37" s="4" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="G37" s="5" t="inlineStr">
+      <c r="H37" s="5" t="inlineStr">
         <is>
           <t>需会视频剪辑（Pr/达芬奇等）、DSLR/微单</t>
         </is>
@@ -34603,25 +34734,30 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
+          <t>学位审核、数据处理</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
           <t>教务注册办公室</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="E38" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="F38" s="4" t="inlineStr">
         <is>
           <t>$20</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="G38" s="4" t="inlineStr">
         <is>
           <t>2026-09-07</t>
         </is>
       </c>
-      <c r="G38" s="5" t="inlineStr">
+      <c r="H38" s="5" t="inlineStr">
         <is>
           <t>需经验；需本科学历 + 1 年相关经验</t>
         </is>
@@ -34638,25 +34774,30 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
+          <t>停车执法</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
           <t>通勤服务</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="E39" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="F39" s="4" t="inlineStr">
         <is>
           <t>$18</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr">
+      <c r="G39" s="4" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="G39" s="5" t="inlineStr">
+      <c r="H39" s="5" t="inlineStr">
         <is>
           <t>需驾照；需经验</t>
         </is>
@@ -34673,25 +34814,30 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
+          <t>学业辅导</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
           <t>体育部</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="E40" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
+      <c r="F40" s="4" t="inlineStr">
         <is>
           <t>$11</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr">
+      <c r="G40" s="4" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="G40" s="5" t="inlineStr">
+      <c r="H40" s="5" t="inlineStr">
         <is>
           <t>需经验；需通过 BCI 背景调查</t>
         </is>
@@ -34708,25 +34854,30 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
+          <t>活动运营</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
           <t>校园商店</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="E41" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="F41" s="4" t="inlineStr">
         <is>
           <t>$18</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr">
+      <c r="G41" s="4" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="G41" s="5" t="inlineStr">
+      <c r="H41" s="5" t="inlineStr">
         <is>
           <t>需驾照</t>
         </is>
@@ -34741,27 +34892,28 @@
           <t>招生办公室学生文员</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="C42" s="5" t="inlineStr"/>
+      <c r="D42" s="5" t="inlineStr">
         <is>
           <t>招生办公室</t>
         </is>
       </c>
-      <c r="D42" s="4" t="inlineStr">
+      <c r="E42" s="4" t="inlineStr">
         <is>
           <t>15-19 hours weekly</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
+      <c r="F42" s="4" t="inlineStr">
         <is>
           <t>$14</t>
         </is>
       </c>
-      <c r="F42" s="4" t="inlineStr">
+      <c r="G42" s="4" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="G42" s="5" t="inlineStr"/>
+      <c r="H42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
@@ -34772,27 +34924,28 @@
           <t>学生住宿大使</t>
         </is>
       </c>
-      <c r="C43" s="5" t="inlineStr">
+      <c r="C43" s="5" t="inlineStr"/>
+      <c r="D43" s="5" t="inlineStr">
         <is>
           <t>住宿与居住教育</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="E43" s="4" t="inlineStr">
         <is>
           <t>19.99</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
+      <c r="F43" s="4" t="inlineStr">
         <is>
           <t>$14</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr">
+      <c r="G43" s="4" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="G43" s="5" t="inlineStr"/>
+      <c r="H43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n">
@@ -34805,25 +34958,30 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
+          <t>社交媒体运营</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
           <t>商业、健康与繁荣中心</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="E44" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="F44" s="4" t="inlineStr">
         <is>
           <t>$14</t>
         </is>
       </c>
-      <c r="F44" s="4" t="inlineStr">
+      <c r="G44" s="4" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="G44" s="5" t="inlineStr"/>
+      <c r="H44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -34834,27 +34992,28 @@
           <t>建筑与规划学院学生大使</t>
         </is>
       </c>
-      <c r="C45" s="5" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr"/>
+      <c r="D45" s="5" t="inlineStr">
         <is>
           <t>建筑与规划学院</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="E45" s="4" t="inlineStr">
         <is>
           <t>8-12</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
+      <c r="F45" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F45" s="4" t="inlineStr">
+      <c r="G45" s="4" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="G45" s="5" t="inlineStr"/>
+      <c r="H45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n">
@@ -34865,27 +35024,28 @@
           <t>活动支持专员</t>
         </is>
       </c>
-      <c r="C46" s="5" t="inlineStr">
+      <c r="C46" s="5" t="inlineStr"/>
+      <c r="D46" s="5" t="inlineStr">
         <is>
           <t>Red Butte 植物园</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="E46" s="4" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="F46" s="4" t="inlineStr">
         <is>
           <t>$15.5</t>
         </is>
       </c>
-      <c r="F46" s="4" t="inlineStr">
+      <c r="G46" s="4" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="G46" s="5" t="inlineStr">
+      <c r="H46" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -34900,27 +35060,28 @@
           <t>办公室与课堂支持助理</t>
         </is>
       </c>
-      <c r="C47" s="5" t="inlineStr">
+      <c r="C47" s="5" t="inlineStr"/>
+      <c r="D47" s="5" t="inlineStr">
         <is>
           <t>高管教育</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr">
+      <c r="E47" s="4" t="inlineStr">
         <is>
           <t>10–19 hours per week, with the potential for increased hours during the summer.</t>
         </is>
       </c>
-      <c r="E47" s="4" t="inlineStr">
+      <c r="F47" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F47" s="4" t="inlineStr">
+      <c r="G47" s="4" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="G47" s="5" t="inlineStr"/>
+      <c r="H47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n">
@@ -34931,27 +35092,28 @@
           <t>国际学生与学者服务同伴助理</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="C48" s="5" t="inlineStr"/>
+      <c r="D48" s="5" t="inlineStr">
         <is>
           <t>国际学生与学者服务中心</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="E48" s="4" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="F48" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F48" s="4" t="inlineStr">
+      <c r="G48" s="4" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="G48" s="5" t="inlineStr"/>
+      <c r="H48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n">
@@ -34964,25 +35126,30 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
+          <t>系统管理、脚本</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
           <t>Marriott 图书馆运营</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr">
+      <c r="E49" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E49" s="4" t="inlineStr">
+      <c r="F49" s="4" t="inlineStr">
         <is>
           <t>$16</t>
         </is>
       </c>
-      <c r="F49" s="4" t="inlineStr">
+      <c r="G49" s="4" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="G49" s="5" t="inlineStr">
+      <c r="H49" s="5" t="inlineStr">
         <is>
           <t>需熟悉 Jamf Pro / SCCM，会脚本（Bash/PowerShell/Python/C/C++）</t>
         </is>
@@ -34999,25 +35166,30 @@
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
+          <t>数据治理、传播</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
           <t>大学分析与机构报告</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
+      <c r="E50" s="4" t="inlineStr">
         <is>
           <t>19 hours</t>
         </is>
       </c>
-      <c r="E50" s="4" t="inlineStr">
+      <c r="F50" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F50" s="4" t="inlineStr">
+      <c r="G50" s="4" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="G50" s="5" t="inlineStr"/>
+      <c r="H50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
@@ -35030,25 +35202,30 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
+          <t>数据治理、技术</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
           <t>大学分析与机构报告</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr">
+      <c r="E51" s="4" t="inlineStr">
         <is>
           <t>19 hours per week</t>
         </is>
       </c>
-      <c r="E51" s="4" t="inlineStr">
+      <c r="F51" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F51" s="4" t="inlineStr">
+      <c r="G51" s="4" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="G51" s="5" t="inlineStr"/>
+      <c r="H51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="n">
@@ -35059,27 +35236,28 @@
           <t>酒店夜班前台文员</t>
         </is>
       </c>
-      <c r="C52" s="5" t="inlineStr">
+      <c r="C52" s="5" t="inlineStr"/>
+      <c r="D52" s="5" t="inlineStr">
         <is>
           <t>大学宾馆</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr">
+      <c r="E52" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E52" s="4" t="inlineStr">
+      <c r="F52" s="4" t="inlineStr">
         <is>
           <t>$19</t>
         </is>
       </c>
-      <c r="F52" s="4" t="inlineStr">
+      <c r="G52" s="4" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="G52" s="5" t="inlineStr">
+      <c r="H52" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -35094,27 +35272,28 @@
           <t>兼职保洁员</t>
         </is>
       </c>
-      <c r="C53" s="5" t="inlineStr">
+      <c r="C53" s="5" t="inlineStr"/>
+      <c r="D53" s="5" t="inlineStr">
         <is>
           <t>住宿与居住教育</t>
         </is>
       </c>
-      <c r="D53" s="4" t="inlineStr">
+      <c r="E53" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="E53" s="4" t="inlineStr">
+      <c r="F53" s="4" t="inlineStr">
         <is>
           <t>$16.16</t>
         </is>
       </c>
-      <c r="F53" s="4" t="inlineStr">
+      <c r="G53" s="4" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>
       </c>
-      <c r="G53" s="5" t="inlineStr"/>
+      <c r="H53" s="5" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n">
@@ -35127,25 +35306,30 @@
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
+          <t>酒水服务</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
           <t>Rice-Eccles 体育场</t>
         </is>
       </c>
-      <c r="D54" s="4" t="inlineStr">
+      <c r="E54" s="4" t="inlineStr">
         <is>
           <t>10-15</t>
         </is>
       </c>
-      <c r="E54" s="4" t="inlineStr">
+      <c r="F54" s="4" t="inlineStr">
         <is>
           <t>$19</t>
         </is>
       </c>
-      <c r="F54" s="4" t="inlineStr">
+      <c r="G54" s="4" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="G54" s="5" t="inlineStr">
+      <c r="H54" s="5" t="inlineStr">
         <is>
           <t>年满 21 岁、需酒类服务证</t>
         </is>
@@ -35160,27 +35344,28 @@
           <t>SCIF 可持续发展大使</t>
         </is>
       </c>
-      <c r="C55" s="5" t="inlineStr">
+      <c r="C55" s="5" t="inlineStr"/>
+      <c r="D55" s="5" t="inlineStr">
         <is>
           <t>可持续校园倡议基金</t>
         </is>
       </c>
-      <c r="D55" s="4" t="inlineStr">
+      <c r="E55" s="4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E55" s="4" t="inlineStr">
+      <c r="F55" s="4" t="inlineStr">
         <is>
           <t>$16</t>
         </is>
       </c>
-      <c r="F55" s="4" t="inlineStr">
+      <c r="G55" s="4" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="G55" s="5" t="inlineStr"/>
+      <c r="H55" s="5" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="n">
@@ -35191,27 +35376,28 @@
           <t>实践学习可持续发展大使</t>
         </is>
       </c>
-      <c r="C56" s="5" t="inlineStr">
+      <c r="C56" s="5" t="inlineStr"/>
+      <c r="D56" s="5" t="inlineStr">
         <is>
           <t>可持续校园倡议基金</t>
         </is>
       </c>
-      <c r="D56" s="4" t="inlineStr">
+      <c r="E56" s="4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E56" s="4" t="inlineStr">
+      <c r="F56" s="4" t="inlineStr">
         <is>
           <t>$16</t>
         </is>
       </c>
-      <c r="F56" s="4" t="inlineStr">
+      <c r="G56" s="4" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="G56" s="5" t="inlineStr"/>
+      <c r="H56" s="5" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n">
@@ -35222,27 +35408,28 @@
           <t>电子与计算机工程系行政助理</t>
         </is>
       </c>
-      <c r="C57" s="5" t="inlineStr">
+      <c r="C57" s="5" t="inlineStr"/>
+      <c r="D57" s="5" t="inlineStr">
         <is>
           <t>电子与计算机工程系</t>
         </is>
       </c>
-      <c r="D57" s="4" t="inlineStr">
+      <c r="E57" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E57" s="4" t="inlineStr">
+      <c r="F57" s="4" t="inlineStr">
         <is>
           <t>$7.25</t>
         </is>
       </c>
-      <c r="F57" s="4" t="inlineStr">
+      <c r="G57" s="4" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="G57" s="5" t="inlineStr"/>
+      <c r="H57" s="5" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="n">
@@ -35255,25 +35442,30 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
+          <t>餐饮技术</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
           <t>Rice-Eccles 体育场</t>
         </is>
       </c>
-      <c r="D58" s="4" t="inlineStr">
+      <c r="E58" s="4" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="E58" s="4" t="inlineStr">
+      <c r="F58" s="4" t="inlineStr">
         <is>
           <t>$16</t>
         </is>
       </c>
-      <c r="F58" s="4" t="inlineStr">
+      <c r="G58" s="4" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="G58" s="5" t="inlineStr">
+      <c r="H58" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -35290,25 +35482,30 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
+          <t>社交媒体运营</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
           <t>多学科设计系</t>
         </is>
       </c>
-      <c r="D59" s="4" t="inlineStr">
+      <c r="E59" s="4" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="E59" s="4" t="inlineStr">
+      <c r="F59" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F59" s="4" t="inlineStr">
+      <c r="G59" s="4" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="G59" s="5" t="inlineStr"/>
+      <c r="H59" s="5" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="n">
@@ -35321,25 +35518,30 @@
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
+          <t>项目支持</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
           <t>本科生教育倡导项目</t>
         </is>
       </c>
-      <c r="D60" s="4" t="inlineStr">
+      <c r="E60" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E60" s="4" t="inlineStr">
+      <c r="F60" s="4" t="inlineStr">
         <is>
           <t>$25</t>
         </is>
       </c>
-      <c r="F60" s="4" t="inlineStr">
+      <c r="G60" s="4" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="G60" s="5" t="inlineStr">
+      <c r="H60" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -35356,25 +35558,30 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
+          <t>舞台管理</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
           <t>音乐学院</t>
         </is>
       </c>
-      <c r="D61" s="4" t="inlineStr">
+      <c r="E61" s="4" t="inlineStr">
         <is>
           <t>Varries based on performance/event schedule</t>
         </is>
       </c>
-      <c r="E61" s="4" t="inlineStr">
+      <c r="F61" s="4" t="inlineStr">
         <is>
           <t>$13</t>
         </is>
       </c>
-      <c r="F61" s="4" t="inlineStr">
+      <c r="G61" s="4" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="G61" s="5" t="inlineStr">
+      <c r="H61" s="5" t="inlineStr">
         <is>
           <t>需经验；需 2 年剧场舞台技术经验</t>
         </is>
@@ -35391,25 +35598,30 @@
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
+          <t>职业咨询</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
           <t>高管教育</t>
         </is>
       </c>
-      <c r="D62" s="4" t="inlineStr">
+      <c r="E62" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E62" s="4" t="inlineStr">
+      <c r="F62" s="4" t="inlineStr">
         <is>
           <t>$30</t>
         </is>
       </c>
-      <c r="F62" s="4" t="inlineStr">
+      <c r="G62" s="4" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="G62" s="5" t="inlineStr">
+      <c r="H62" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -35426,25 +35638,30 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
+          <t>市场营销、设计</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
           <t>学生会</t>
         </is>
       </c>
-      <c r="D63" s="4" t="inlineStr">
+      <c r="E63" s="4" t="inlineStr">
         <is>
           <t>up to 19 hours/week</t>
         </is>
       </c>
-      <c r="E63" s="4" t="inlineStr">
+      <c r="F63" s="4" t="inlineStr">
         <is>
           <t>$14</t>
         </is>
       </c>
-      <c r="F63" s="4" t="inlineStr">
+      <c r="G63" s="4" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="G63" s="5" t="inlineStr"/>
+      <c r="H63" s="5" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="4" t="n">
@@ -35455,27 +35672,28 @@
           <t>Utech 技术服务助理</t>
         </is>
       </c>
-      <c r="C64" s="5" t="inlineStr">
+      <c r="C64" s="5" t="inlineStr"/>
+      <c r="D64" s="5" t="inlineStr">
         <is>
           <t>校园商店</t>
         </is>
       </c>
-      <c r="D64" s="4" t="inlineStr">
+      <c r="E64" s="4" t="inlineStr">
         <is>
           <t>19-20</t>
         </is>
       </c>
-      <c r="E64" s="4" t="inlineStr">
+      <c r="F64" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F64" s="4" t="inlineStr">
+      <c r="G64" s="4" t="inlineStr">
         <is>
           <t>2026-10-03</t>
         </is>
       </c>
-      <c r="G64" s="5" t="inlineStr">
+      <c r="H64" s="5" t="inlineStr">
         <is>
           <t>需通过安全审查（security clearance）</t>
         </is>
@@ -35490,27 +35708,28 @@
           <t>订单履约助理</t>
         </is>
       </c>
-      <c r="C65" s="5" t="inlineStr">
+      <c r="C65" s="5" t="inlineStr"/>
+      <c r="D65" s="5" t="inlineStr">
         <is>
           <t>校园商店</t>
         </is>
       </c>
-      <c r="D65" s="4" t="inlineStr">
+      <c r="E65" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="E65" s="4" t="inlineStr">
+      <c r="F65" s="4" t="inlineStr">
         <is>
           <t>$14.5</t>
         </is>
       </c>
-      <c r="F65" s="4" t="inlineStr">
+      <c r="G65" s="4" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="G65" s="5" t="inlineStr"/>
+      <c r="H65" s="5" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="n">
@@ -35523,25 +35742,30 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
+          <t>体育裁判</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
           <t>校内体育</t>
         </is>
       </c>
-      <c r="D66" s="4" t="inlineStr">
+      <c r="E66" s="4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E66" s="4" t="inlineStr">
+      <c r="F66" s="4" t="inlineStr">
         <is>
           <t>$12</t>
         </is>
       </c>
-      <c r="F66" s="4" t="inlineStr">
+      <c r="G66" s="4" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>
       </c>
-      <c r="G66" s="5" t="inlineStr">
+      <c r="H66" s="5" t="inlineStr">
         <is>
           <t>需 CPR 认证（可入职一月内取得）</t>
         </is>
@@ -35556,27 +35780,28 @@
           <t>仓库工作人员</t>
         </is>
       </c>
-      <c r="C67" s="5" t="inlineStr">
+      <c r="C67" s="5" t="inlineStr"/>
+      <c r="D67" s="5" t="inlineStr">
         <is>
           <t>Rice-Eccles 体育场</t>
         </is>
       </c>
-      <c r="D67" s="4" t="inlineStr">
+      <c r="E67" s="4" t="inlineStr">
         <is>
           <t>4 hours per week or less</t>
         </is>
       </c>
-      <c r="E67" s="4" t="inlineStr">
+      <c r="F67" s="4" t="inlineStr">
         <is>
           <t>$16</t>
         </is>
       </c>
-      <c r="F67" s="4" t="inlineStr">
+      <c r="G67" s="4" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="G67" s="5" t="inlineStr">
+      <c r="H67" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -35591,27 +35816,28 @@
           <t>体育场餐饮售卖人员</t>
         </is>
       </c>
-      <c r="C68" s="5" t="inlineStr">
+      <c r="C68" s="5" t="inlineStr"/>
+      <c r="D68" s="5" t="inlineStr">
         <is>
           <t>Rice-Eccles 体育场</t>
         </is>
       </c>
-      <c r="D68" s="4" t="inlineStr">
+      <c r="E68" s="4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E68" s="4" t="inlineStr">
+      <c r="F68" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F68" s="4" t="inlineStr">
+      <c r="G68" s="4" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="G68" s="5" t="inlineStr">
+      <c r="H68" s="5" t="inlineStr">
         <is>
           <t>需食品证</t>
         </is>
@@ -35626,27 +35852,28 @@
           <t>兼职保洁员</t>
         </is>
       </c>
-      <c r="C69" s="5" t="inlineStr">
+      <c r="C69" s="5" t="inlineStr"/>
+      <c r="D69" s="5" t="inlineStr">
         <is>
           <t>住宿与居住教育</t>
         </is>
       </c>
-      <c r="D69" s="4" t="inlineStr">
+      <c r="E69" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E69" s="4" t="inlineStr">
+      <c r="F69" s="4" t="inlineStr">
         <is>
           <t>$16.16</t>
         </is>
       </c>
-      <c r="F69" s="4" t="inlineStr">
+      <c r="G69" s="4" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="G69" s="5" t="inlineStr"/>
+      <c r="H69" s="5" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="4" t="n">
@@ -35659,25 +35886,30 @@
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
+          <t>后厨</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
           <t>犹他美术博物馆</t>
         </is>
       </c>
-      <c r="D70" s="4" t="inlineStr">
+      <c r="E70" s="4" t="inlineStr">
         <is>
           <t>1-19</t>
         </is>
       </c>
-      <c r="E70" s="4" t="inlineStr">
+      <c r="F70" s="4" t="inlineStr">
         <is>
           <t>$14</t>
         </is>
       </c>
-      <c r="F70" s="4" t="inlineStr">
+      <c r="G70" s="4" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="G70" s="5" t="inlineStr">
+      <c r="H70" s="5" t="inlineStr">
         <is>
           <t>需食品证</t>
         </is>
@@ -35692,27 +35924,28 @@
           <t>UMFA 商店店员</t>
         </is>
       </c>
-      <c r="C71" s="5" t="inlineStr">
+      <c r="C71" s="5" t="inlineStr"/>
+      <c r="D71" s="5" t="inlineStr">
         <is>
           <t>犹他美术博物馆</t>
         </is>
       </c>
-      <c r="D71" s="4" t="inlineStr">
+      <c r="E71" s="4" t="inlineStr">
         <is>
           <t>1-19</t>
         </is>
       </c>
-      <c r="E71" s="4" t="inlineStr">
+      <c r="F71" s="4" t="inlineStr">
         <is>
           <t>$13.65</t>
         </is>
       </c>
-      <c r="F71" s="4" t="inlineStr">
+      <c r="G71" s="4" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="G71" s="5" t="inlineStr">
+      <c r="H71" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -35729,25 +35962,30 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
+          <t>驾驶、安保</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
           <t>通勤服务</t>
         </is>
       </c>
-      <c r="D72" s="4" t="inlineStr">
+      <c r="E72" s="4" t="inlineStr">
         <is>
           <t>15-19 hours per week</t>
         </is>
       </c>
-      <c r="E72" s="4" t="inlineStr">
+      <c r="F72" s="4" t="inlineStr">
         <is>
           <t>$15.38</t>
         </is>
       </c>
-      <c r="F72" s="4" t="inlineStr">
+      <c r="G72" s="4" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="G72" s="5" t="inlineStr">
+      <c r="H72" s="5" t="inlineStr">
         <is>
           <t>需驾照</t>
         </is>
@@ -35762,27 +36000,28 @@
           <t>顾客服务代表</t>
         </is>
       </c>
-      <c r="C73" s="5" t="inlineStr">
+      <c r="C73" s="5" t="inlineStr"/>
+      <c r="D73" s="5" t="inlineStr">
         <is>
           <t>财务与运营</t>
         </is>
       </c>
-      <c r="D73" s="4" t="inlineStr">
+      <c r="E73" s="4" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="E73" s="4" t="inlineStr">
+      <c r="F73" s="4" t="inlineStr">
         <is>
           <t>$16</t>
         </is>
       </c>
-      <c r="F73" s="4" t="inlineStr">
+      <c r="G73" s="4" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G73" s="5" t="inlineStr">
+      <c r="H73" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -35799,25 +36038,30 @@
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
+          <t>活动支持</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
           <t>犹他美术博物馆</t>
         </is>
       </c>
-      <c r="D74" s="4" t="inlineStr">
+      <c r="E74" s="4" t="inlineStr">
         <is>
           <t>0-19</t>
         </is>
       </c>
-      <c r="E74" s="4" t="inlineStr">
+      <c r="F74" s="4" t="inlineStr">
         <is>
           <t>$13.65</t>
         </is>
       </c>
-      <c r="F74" s="4" t="inlineStr">
+      <c r="G74" s="4" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G74" s="5" t="inlineStr">
+      <c r="H74" s="5" t="inlineStr">
         <is>
           <t>需经验；能提举 50 磅</t>
         </is>
@@ -35834,25 +36078,30 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
+          <t>驾驶</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
           <t>通勤服务</t>
         </is>
       </c>
-      <c r="D75" s="4" t="inlineStr">
+      <c r="E75" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="E75" s="4" t="inlineStr">
+      <c r="F75" s="4" t="inlineStr">
         <is>
           <t>$20</t>
         </is>
       </c>
-      <c r="F75" s="4" t="inlineStr">
+      <c r="G75" s="4" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="G75" s="5" t="inlineStr">
+      <c r="H75" s="5" t="inlineStr">
         <is>
           <t>需 CDL 驾照（提供付费培训）</t>
         </is>
@@ -35867,27 +36116,28 @@
           <t>兼职保洁员</t>
         </is>
       </c>
-      <c r="C76" s="5" t="inlineStr">
+      <c r="C76" s="5" t="inlineStr"/>
+      <c r="D76" s="5" t="inlineStr">
         <is>
           <t>住宿与居住教育</t>
         </is>
       </c>
-      <c r="D76" s="4" t="inlineStr">
+      <c r="E76" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E76" s="4" t="inlineStr">
+      <c r="F76" s="4" t="inlineStr">
         <is>
           <t>$16.16</t>
         </is>
       </c>
-      <c r="F76" s="4" t="inlineStr">
+      <c r="G76" s="4" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="G76" s="5" t="inlineStr"/>
+      <c r="H76" s="5" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="n">
@@ -35900,25 +36150,30 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
+          <t>市场营销</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
           <t>校园健康中心</t>
         </is>
       </c>
-      <c r="D77" s="4" t="inlineStr">
+      <c r="E77" s="4" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="E77" s="4" t="inlineStr">
+      <c r="F77" s="4" t="inlineStr">
         <is>
           <t>$14.5</t>
         </is>
       </c>
-      <c r="F77" s="4" t="inlineStr">
+      <c r="G77" s="4" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="G77" s="5" t="inlineStr"/>
+      <c r="H77" s="5" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="n">
@@ -35929,27 +36184,28 @@
           <t>教材与课程资料助理</t>
         </is>
       </c>
-      <c r="C78" s="5" t="inlineStr">
+      <c r="C78" s="5" t="inlineStr"/>
+      <c r="D78" s="5" t="inlineStr">
         <is>
           <t>校园商店</t>
         </is>
       </c>
-      <c r="D78" s="4" t="inlineStr">
+      <c r="E78" s="4" t="inlineStr">
         <is>
           <t>19-20</t>
         </is>
       </c>
-      <c r="E78" s="4" t="inlineStr">
+      <c r="F78" s="4" t="inlineStr">
         <is>
           <t>$14.5</t>
         </is>
       </c>
-      <c r="F78" s="4" t="inlineStr">
+      <c r="G78" s="4" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="G78" s="5" t="inlineStr"/>
+      <c r="H78" s="5" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="n">
@@ -35960,27 +36216,28 @@
           <t>UMFA 安保服务人员</t>
         </is>
       </c>
-      <c r="C79" s="5" t="inlineStr">
+      <c r="C79" s="5" t="inlineStr"/>
+      <c r="D79" s="5" t="inlineStr">
         <is>
           <t>犹他美术博物馆</t>
         </is>
       </c>
-      <c r="D79" s="4" t="inlineStr">
+      <c r="E79" s="4" t="inlineStr">
         <is>
           <t>1-19</t>
         </is>
       </c>
-      <c r="E79" s="4" t="inlineStr">
+      <c r="F79" s="4" t="inlineStr">
         <is>
           <t>$13.65</t>
         </is>
       </c>
-      <c r="F79" s="4" t="inlineStr">
+      <c r="G79" s="4" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="G79" s="5" t="inlineStr">
+      <c r="H79" s="5" t="inlineStr">
         <is>
           <t>需驾照；需经验；需通过背景调查</t>
         </is>
@@ -35995,27 +36252,28 @@
           <t>Wilkes 中心学生大使</t>
         </is>
       </c>
-      <c r="C80" s="5" t="inlineStr">
+      <c r="C80" s="5" t="inlineStr"/>
+      <c r="D80" s="5" t="inlineStr">
         <is>
           <t>Wilkes 气候科学与政策中心</t>
         </is>
       </c>
-      <c r="D80" s="4" t="inlineStr">
+      <c r="E80" s="4" t="inlineStr">
         <is>
           <t>10-15</t>
         </is>
       </c>
-      <c r="E80" s="4" t="inlineStr">
+      <c r="F80" s="4" t="inlineStr">
         <is>
           <t>$14</t>
         </is>
       </c>
-      <c r="F80" s="4" t="inlineStr">
+      <c r="G80" s="4" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="G80" s="5" t="inlineStr"/>
+      <c r="H80" s="5" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="n">
@@ -36026,27 +36284,28 @@
           <t>实验室助理</t>
         </is>
       </c>
-      <c r="C81" s="5" t="inlineStr">
+      <c r="C81" s="5" t="inlineStr"/>
+      <c r="D81" s="5" t="inlineStr">
         <is>
           <t>Huntsman 癌症研究所·Chandrasekharan 实验室</t>
         </is>
       </c>
-      <c r="D81" s="4" t="inlineStr">
+      <c r="E81" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="E81" s="4" t="inlineStr">
+      <c r="F81" s="4" t="inlineStr">
         <is>
           <t>$7.25</t>
         </is>
       </c>
-      <c r="F81" s="4" t="inlineStr">
+      <c r="G81" s="4" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="G81" s="5" t="inlineStr"/>
+      <c r="H81" s="5" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="n">
@@ -36057,27 +36316,28 @@
           <t>前厅收银员</t>
         </is>
       </c>
-      <c r="C82" s="5" t="inlineStr">
+      <c r="C82" s="5" t="inlineStr"/>
+      <c r="D82" s="5" t="inlineStr">
         <is>
           <t>先锋剧院</t>
         </is>
       </c>
-      <c r="D82" s="4" t="inlineStr">
+      <c r="E82" s="4" t="inlineStr">
         <is>
           <t>15-20</t>
         </is>
       </c>
-      <c r="E82" s="4" t="inlineStr">
+      <c r="F82" s="4" t="inlineStr">
         <is>
           <t>$11</t>
         </is>
       </c>
-      <c r="F82" s="4" t="inlineStr">
+      <c r="G82" s="4" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="G82" s="5" t="inlineStr">
+      <c r="H82" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -36092,27 +36352,28 @@
           <t>票房售票员</t>
         </is>
       </c>
-      <c r="C83" s="5" t="inlineStr">
+      <c r="C83" s="5" t="inlineStr"/>
+      <c r="D83" s="5" t="inlineStr">
         <is>
           <t>先锋剧院</t>
         </is>
       </c>
-      <c r="D83" s="4" t="inlineStr">
+      <c r="E83" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="E83" s="4" t="inlineStr">
+      <c r="F83" s="4" t="inlineStr">
         <is>
           <t>$10.5</t>
         </is>
       </c>
-      <c r="F83" s="4" t="inlineStr">
+      <c r="G83" s="4" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="G83" s="5" t="inlineStr">
+      <c r="H83" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -36127,27 +36388,28 @@
           <t>行政文员</t>
         </is>
       </c>
-      <c r="C84" s="5" t="inlineStr">
+      <c r="C84" s="5" t="inlineStr"/>
+      <c r="D84" s="5" t="inlineStr">
         <is>
           <t>校园卡服务</t>
         </is>
       </c>
-      <c r="D84" s="4" t="inlineStr">
+      <c r="E84" s="4" t="inlineStr">
         <is>
           <t>15-19 hours per week</t>
         </is>
       </c>
-      <c r="E84" s="4" t="inlineStr">
+      <c r="F84" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="F84" s="4" t="inlineStr">
+      <c r="G84" s="4" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="G84" s="5" t="inlineStr">
+      <c r="H84" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -36164,25 +36426,30 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
+          <t>舞台技术</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
           <t>UtahPresents 演出项目</t>
         </is>
       </c>
-      <c r="D85" s="4" t="inlineStr">
+      <c r="E85" s="4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E85" s="4" t="inlineStr">
+      <c r="F85" s="4" t="inlineStr">
         <is>
           <t>$16</t>
         </is>
       </c>
-      <c r="F85" s="4" t="inlineStr">
+      <c r="G85" s="4" t="inlineStr">
         <is>
           <t>2026-11-05</t>
         </is>
       </c>
-      <c r="G85" s="5" t="inlineStr">
+      <c r="H85" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -36197,27 +36464,28 @@
           <t>网球中心前台工作人员</t>
         </is>
       </c>
-      <c r="C86" s="5" t="inlineStr">
+      <c r="C86" s="5" t="inlineStr"/>
+      <c r="D86" s="5" t="inlineStr">
         <is>
           <t>体育部</t>
         </is>
       </c>
-      <c r="D86" s="4" t="inlineStr">
+      <c r="E86" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E86" s="4" t="inlineStr">
+      <c r="F86" s="4" t="inlineStr">
         <is>
           <t>$7.25</t>
         </is>
       </c>
-      <c r="F86" s="4" t="inlineStr">
+      <c r="G86" s="4" t="inlineStr">
         <is>
           <t>2026-11-07</t>
         </is>
       </c>
-      <c r="G86" s="5" t="inlineStr"/>
+      <c r="H86" s="5" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="n">
@@ -36230,25 +36498,30 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
+          <t>TESOL 教学</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
           <t>英语语言学院</t>
         </is>
       </c>
-      <c r="D87" s="4" t="inlineStr">
+      <c r="E87" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="E87" s="4" t="inlineStr">
+      <c r="F87" s="4" t="inlineStr">
         <is>
           <t>$49</t>
         </is>
       </c>
-      <c r="F87" s="4" t="inlineStr">
+      <c r="G87" s="4" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="G87" s="5" t="inlineStr">
+      <c r="H87" s="5" t="inlineStr">
         <is>
           <t>需 TESOL 硕士 + TESOL 证书</t>
         </is>
@@ -36263,27 +36536,28 @@
           <t>住宿招生与外联协调员</t>
         </is>
       </c>
-      <c r="C88" s="5" t="inlineStr">
+      <c r="C88" s="5" t="inlineStr"/>
+      <c r="D88" s="5" t="inlineStr">
         <is>
           <t>影响力与繁荣中心</t>
         </is>
       </c>
-      <c r="D88" s="4" t="inlineStr">
+      <c r="E88" s="4" t="inlineStr">
         <is>
           <t>15-19</t>
         </is>
       </c>
-      <c r="E88" s="4" t="inlineStr">
+      <c r="F88" s="4" t="inlineStr">
         <is>
           <t>$12</t>
         </is>
       </c>
-      <c r="F88" s="4" t="inlineStr">
+      <c r="G88" s="4" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="G88" s="5" t="inlineStr"/>
+      <c r="H88" s="5" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="n">
@@ -36296,25 +36570,30 @@
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
+          <t>摄像</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
           <t>舞蹈学院</t>
         </is>
       </c>
-      <c r="D89" s="4" t="inlineStr">
+      <c r="E89" s="4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E89" s="4" t="inlineStr">
+      <c r="F89" s="4" t="inlineStr">
         <is>
           <t>$13.5</t>
         </is>
       </c>
-      <c r="F89" s="4" t="inlineStr">
+      <c r="G89" s="4" t="inlineStr">
         <is>
           <t>2026-12-31</t>
         </is>
       </c>
-      <c r="G89" s="5" t="inlineStr"/>
+      <c r="H89" s="5" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="n">
@@ -36327,31 +36606,36 @@
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
+          <t>舞台技术</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
           <t>舞蹈学院</t>
         </is>
       </c>
-      <c r="D90" s="4" t="inlineStr">
+      <c r="E90" s="4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E90" s="4" t="inlineStr">
+      <c r="F90" s="4" t="inlineStr">
         <is>
           <t>$13.5</t>
         </is>
       </c>
-      <c r="F90" s="4" t="inlineStr">
+      <c r="G90" s="4" t="inlineStr">
         <is>
           <t>2026-12-31</t>
         </is>
       </c>
-      <c r="G90" s="5" t="inlineStr"/>
+      <c r="H90" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G90"/>
+  <autoFilter ref="A4:H90"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId1"/>

</xml_diff>

<commit_message>
Add job-content column and clarify 26Fall timeframe in intl sheet
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'岗位检索'!$A$4:$W$126</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'MEAE国际学生省流版'!$A$4:$H$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'MEAE国际学生省流版'!$A$4:$I$90</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33421,17 +33421,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H90"/>
+  <dimension ref="A1:I90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -33444,7 +33445,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>面向 MEAE 硕士国际学生（F-1）· 已排除 36 个必须勤工助学、仅限本科、已关闭或需公民身份的岗位 · 快照 2026-08-16T05:02:08.919027+08:00</t>
+          <t>面向 26Fall（2026 秋季学期）校内兼职 · 快照 2026-08-16 · 2026-08-17 及之后申请适用 · 已排除 36 个（勤工助学必需 / 仅限本科 / 已关闭 / 需公民身份）</t>
         </is>
       </c>
     </row>
@@ -33467,25 +33468,30 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
+          <t>工作内容</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
           <t>部门</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>每周工时</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>时薪</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>截止日期</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>注意</t>
         </is>
@@ -33507,25 +33513,30 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
+          <t>在 University Information Technology（UIT）下属 University Suppor…</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
           <t>大学信息技术部·校级支持服务</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr"/>
+      <c r="I5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -33543,25 +33554,30 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
+          <t>为现场和远程员工处理基础或一级 IT、视听问题，包括台式机、笔记本电脑和网络服务</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
           <t>犹他自然历史博物馆</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>$17</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -33583,25 +33599,30 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
+          <t>Yitong Xin 博士招聘一名研究生研究助理（职位代码 1632），支持团队不断增加的研究项目，主题包括迷幻药辅助治…</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
           <t>社会工作学院</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>未提供</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>需社工硕士/博士在读，会 Mplus/SPSS/R</t>
         </is>
@@ -33623,25 +33644,30 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
+          <t>艺术与艺术史系招聘人体艺术模特，需要完成着衣和裸体姿势</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
           <t>艺术与艺术史系</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>0-6</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>$20</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr"/>
+      <c r="I8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -33659,25 +33685,30 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
+          <t>为易损文物、标本和其他藏品设计、制作并安装符合文物保护要求的定制展示支架</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
           <t>犹他自然历史博物馆</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>10-15</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>$35</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>需驾照；需经验</t>
         </is>
@@ -33699,25 +33730,30 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
+          <t>KUER 招聘一名有创意、注重细节的社交媒体助理，每周工作 19 小时，帮助扩大数字平台受众并提高互动</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
           <t>KUER 公共广播电台</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>$17</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -33735,25 +33771,30 @@
       <c r="C11" s="5" t="inlineStr"/>
       <c r="D11" s="5" t="inlineStr">
         <is>
+          <t>在校园商店多个业务区域轮岗，为顾客提供服务，并协助收银、商品陈列、补货和维护卖场</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
           <t>校园商店</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>19-20</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>DOE</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr"/>
+      <c r="I11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -33771,25 +33812,30 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
+          <t>Student Parent Support Center 为犹他大学学生、教职员工和患者提供信息、支持及家庭资源</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
           <t>学生家长支持中心</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>$15.5</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>食品证可后考；需经验；需 CPR/急救证，能抱举幼儿</t>
         </is>
@@ -33811,25 +33857,30 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
+          <t>Student Parent Support Center 为犹他大学学生、教职员工和患者提供信息、支持及家庭资源</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
           <t>学生家长支持中心</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>up to 19 hours/week, depending on hiring needs and incumbent schedule</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>$14.5</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>食品证可后考；入职 60 天内需食品证、TB 检测、BCI 背景调查、急救培训</t>
         </is>
@@ -33851,25 +33902,30 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
+          <t>面向大学生的入门岗位</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
           <t>在线教育</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>$12</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr"/>
+      <c r="I14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -33883,25 +33939,30 @@
       <c r="C15" s="5" t="inlineStr"/>
       <c r="D15" s="5" t="inlineStr">
         <is>
+          <t>犹他大学校园商店招聘兼职收发货班次文员，支持收发货部门的日常运营</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
           <t>校园商店</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>$16</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -33923,25 +33984,30 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
+          <t>世界语言与文化系招聘兼职讲师，在 2026 年秋季学期教授一年级韩语</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
           <t>世界语言与文化系</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>4,200-6,000</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>需驾照；韩语接近母语级</t>
         </is>
@@ -33963,25 +34029,30 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
+          <t>在内容经理指导下协助校友传播和内容制作</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
           <t>校友关系办公室</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>8-10</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr"/>
+      <c r="I17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
@@ -33999,25 +34070,30 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
+          <t>在主管 Emma 的指导下维护校友社交媒体账号，参与内容制作、活动报道和平台管理，重点做好故事表达、用户互动和内容组织</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
           <t>校友关系办公室</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="H18" s="5" t="inlineStr"/>
+      <c r="I18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -34031,25 +34107,30 @@
       <c r="C19" s="5" t="inlineStr"/>
       <c r="D19" s="5" t="inlineStr">
         <is>
+          <t>Eccles Alumni House 招聘兼职活动工作人员，需要具备良好的顾客服务能力并能接受不固定排班</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
           <t>校友关系办公室</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>15-19</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>$15.6</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr"/>
+      <c r="I19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
@@ -34067,25 +34148,30 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
+          <t>协助自然历史博物馆扩大 Research Quest 科学教育项目的全国影响力，主要负责自动化邮件营销、活动数据分析、A…</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
           <t>犹他自然历史博物馆</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>需经验；需本科学历+2年经验 或 硕士</t>
         </is>
@@ -34107,25 +34193,30 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
+          <t>为 MBA 项目教师提供支持，协助制作在线课程材料并进行质量检查，与教师、教学设计师和学生直接合作</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
           <t>高管教育</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>15 to 19</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="I21" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -34143,25 +34234,30 @@
       <c r="C22" s="5" t="inlineStr"/>
       <c r="D22" s="5" t="inlineStr">
         <is>
+          <t>负责 Marriott Library 的设施管理和维护，可独立完成分配的任务，也会与团队共同推进项目，并与不同部门合作…</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
           <t>Marriott 图书馆运营</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>能提举 25 磅、爬梯凳</t>
         </is>
@@ -34179,25 +34275,30 @@
       <c r="C23" s="5" t="inlineStr"/>
       <c r="D23" s="5" t="inlineStr">
         <is>
+          <t>犹他自然历史博物馆招聘一名学生，协助古生物藏品管理和登记工作</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
           <t>犹他自然历史博物馆</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>$15.6</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="H23" s="5" t="inlineStr">
+      <c r="I23" s="5" t="inlineStr">
         <is>
           <t>需经验；需通过背景调查</t>
         </is>
@@ -34219,25 +34320,30 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
+          <t>负责监督犹他大学体育场和竞技馆餐饮服务，确保服务水平和操作标准持续达标；确认员工得到适当培训，并在需要时为他们提供现场协…</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
           <t>Rice-Eccles 体育场</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>16 hours per week or less</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>$18</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="H24" s="5" t="inlineStr">
+      <c r="I24" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -34255,25 +34361,30 @@
       <c r="C25" s="5" t="inlineStr"/>
       <c r="D25" s="5" t="inlineStr">
         <is>
+          <t>为体育设施、活动和运动草坪／场地运营提供一般支持，协助全职员工完成日常维护、活动搭建与撤场、设施保养，以及各体育场馆和户…</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
           <t>体育部</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>$16</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="H25" s="5" t="inlineStr">
+      <c r="I25" s="5" t="inlineStr">
         <is>
           <t>需驾照；需经验；能提举 60 磅、需美国驾照</t>
         </is>
@@ -34295,25 +34406,30 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
+          <t>作为团队成员支持 Bennion Center for Community Engagement 的日常运营和各类项目需…</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
           <t>Bennion 社区参与中心</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>As needed</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="H26" s="5" t="inlineStr"/>
+      <c r="I26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -34327,25 +34443,30 @@
       <c r="C27" s="5" t="inlineStr"/>
       <c r="D27" s="5" t="inlineStr">
         <is>
+          <t>加入 Red Butte Garden and Arboretum 成人项目部门，协助开展健康、创意、园艺、生态和烹饪等…</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
           <t>Red Butte 植物园</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>$16</t>
         </is>
       </c>
-      <c r="G27" s="4" t="inlineStr">
+      <c r="H27" s="4" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="H27" s="5" t="inlineStr">
+      <c r="I27" s="5" t="inlineStr">
         <is>
           <t>需驾照；需经验；能提举 50 磅、走崎岖地形</t>
         </is>
@@ -34363,25 +34484,30 @@
       <c r="C28" s="5" t="inlineStr"/>
       <c r="D28" s="5" t="inlineStr">
         <is>
+          <t>当面或通过电话接待并协助访客，提供一般办公室支持</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
           <t>S.J. Quinney 法学院</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>$9.62</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="H28" s="5" t="inlineStr">
+      <c r="I28" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -34403,25 +34529,30 @@
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
+          <t>Pathway Engineering 团队负责建设和改善犹他大学物理网络层基础设施，包括在校园和医院楼宇内铺设、端接铜…</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
           <t>信息管理</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>15 - 19</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G29" s="4" t="inlineStr">
+      <c r="H29" s="4" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="H29" s="5" t="inlineStr"/>
+      <c r="I29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
@@ -34439,25 +34570,30 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
+          <t>商业、健康与繁荣中心位于 Impact &amp; Prosperity Epicenter，Prosperity U 是其面向…</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
           <t>商业、健康与繁荣中心</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>$12</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr">
+      <c r="H30" s="4" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="H30" s="5" t="inlineStr"/>
+      <c r="I30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -34475,25 +34611,30 @@
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
+          <t>在 Kahlert Village 的 Adobe Creative Commons 担任创意软件顾问，帮助犹他大学师生…</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
           <t>大学信息技术部·数字学习技术</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G31" s="4" t="inlineStr">
+      <c r="H31" s="4" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="H31" s="5" t="inlineStr">
+      <c r="I31" s="5" t="inlineStr">
         <is>
           <t>需精通至少 4 款 Adobe 应用</t>
         </is>
@@ -34515,25 +34656,30 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
+          <t>犹他大学 Student Media &amp; ABD 招聘学生担任办公室副经理</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
           <t>学生媒体委员会</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>15-20</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="G32" s="4" t="inlineStr">
         <is>
           <t>$11</t>
         </is>
       </c>
-      <c r="G32" s="4" t="inlineStr">
+      <c r="H32" s="4" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="H32" s="5" t="inlineStr"/>
+      <c r="I32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -34547,25 +34693,30 @@
       <c r="C33" s="5" t="inlineStr"/>
       <c r="D33" s="5" t="inlineStr">
         <is>
+          <t>Utah Nanofab 招聘一名办公室助理，为员工提供一般行政支持</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
           <t>犹他纳米制造实验室</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="F33" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="G33" s="4" t="inlineStr">
         <is>
           <t>$7.25</t>
         </is>
       </c>
-      <c r="G33" s="4" t="inlineStr">
+      <c r="H33" s="4" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="H33" s="5" t="inlineStr"/>
+      <c r="I33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
@@ -34583,25 +34734,30 @@
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
+          <t>协助策划、执行和评估犹他自然历史博物馆 Critical Action Lab 项目的活动、会议和事件</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
           <t>犹他自然历史博物馆</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="G34" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr">
+      <c r="H34" s="4" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="H34" s="5" t="inlineStr">
+      <c r="I34" s="5" t="inlineStr">
         <is>
           <t>需驾照；需经验；需本科学历、驾照</t>
         </is>
@@ -34619,25 +34775,30 @@
       <c r="C35" s="5" t="inlineStr"/>
       <c r="D35" s="5" t="inlineStr">
         <is>
+          <t>接待酒店来宾，办理入住和退房，并协助处理问题或顾虑；有需要时也会在预订部门帮助客人订房，或支援早餐部门</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
           <t>大学宾馆</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="G35" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G35" s="4" t="inlineStr">
+      <c r="H35" s="4" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="H35" s="5" t="inlineStr">
+      <c r="I35" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -34659,25 +34820,30 @@
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
+          <t>犹他自然历史博物馆（NHMU）的公众项目包括多种馆内活动，用于配合展览和馆藏，帮助访客了解自然世界并与社区建立联系</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
           <t>犹他自然历史博物馆</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="F36" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
+      <c r="G36" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G36" s="4" t="inlineStr">
+      <c r="H36" s="4" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="H36" s="5" t="inlineStr">
+      <c r="I36" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -34699,25 +34865,30 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
+          <t>校友关系办公室招聘视频实习生，为 The Mighty Utah Student Section（MUSS）和 Stud…</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
           <t>校友关系办公室</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="F37" s="4" t="inlineStr">
         <is>
           <t>15-19</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr">
+      <c r="G37" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G37" s="4" t="inlineStr">
+      <c r="H37" s="4" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="H37" s="5" t="inlineStr">
+      <c r="I37" s="5" t="inlineStr">
         <is>
           <t>需会视频剪辑（Pr/达芬奇等）、DSLR/微单</t>
         </is>
@@ -34739,25 +34910,30 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
+          <t>为 Academic Progress 助理注册主任提供课程和学位审核方面的行政及分析支持，重点是通过学位审核确保学生学…</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
           <t>教务注册办公室</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="F38" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="G38" s="4" t="inlineStr">
         <is>
           <t>$20</t>
         </is>
       </c>
-      <c r="G38" s="4" t="inlineStr">
+      <c r="H38" s="4" t="inlineStr">
         <is>
           <t>2026-09-07</t>
         </is>
       </c>
-      <c r="H38" s="5" t="inlineStr">
+      <c r="I38" s="5" t="inlineStr">
         <is>
           <t>需经验；需本科学历 + 1 年相关经验</t>
         </is>
@@ -34779,25 +34955,30 @@
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
+          <t>定期巡查并监督停车区域，处理违规停车，确保车位留给持有效许可的人员和特殊用途访客，同时为犹他大学师生和来访者提供服务</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
           <t>通勤服务</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="F39" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr">
+      <c r="G39" s="4" t="inlineStr">
         <is>
           <t>$18</t>
         </is>
       </c>
-      <c r="G39" s="4" t="inlineStr">
+      <c r="H39" s="4" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="H39" s="5" t="inlineStr">
+      <c r="I39" s="5" t="inlineStr">
         <is>
           <t>需驾照；需经验</t>
         </is>
@@ -34819,25 +35000,30 @@
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
+          <t>为学生提供一对一或小组辅导，定期沟通以找出学习困难、改善学习方法并提高成绩</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
           <t>体育部</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
+      <c r="F40" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr">
+      <c r="G40" s="4" t="inlineStr">
         <is>
           <t>$11</t>
         </is>
       </c>
-      <c r="G40" s="4" t="inlineStr">
+      <c r="H40" s="4" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="H40" s="5" t="inlineStr">
+      <c r="I40" s="5" t="inlineStr">
         <is>
           <t>需经验；需通过 BCI 背景调查</t>
         </is>
@@ -34859,25 +35045,30 @@
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
+          <t>支持犹他大学校园商店在橄榄球比赛、其他体育赛事和校内特别活动中销售官方授权的 Utah Athletics 服装、礼品和…</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
           <t>校园商店</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="F41" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr">
+      <c r="G41" s="4" t="inlineStr">
         <is>
           <t>$18</t>
         </is>
       </c>
-      <c r="G41" s="4" t="inlineStr">
+      <c r="H41" s="4" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="H41" s="5" t="inlineStr">
+      <c r="I41" s="5" t="inlineStr">
         <is>
           <t>需驾照</t>
         </is>
@@ -34895,25 +35086,30 @@
       <c r="C42" s="5" t="inlineStr"/>
       <c r="D42" s="5" t="inlineStr">
         <is>
+          <t>招生办公室招聘学生文员，工作地点包括文件影像处理部门和本科招生材料处理部门</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
           <t>招生办公室</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
+      <c r="F42" s="4" t="inlineStr">
         <is>
           <t>15-19 hours weekly</t>
         </is>
       </c>
-      <c r="F42" s="4" t="inlineStr">
+      <c r="G42" s="4" t="inlineStr">
         <is>
           <t>$14</t>
         </is>
       </c>
-      <c r="G42" s="4" t="inlineStr">
+      <c r="H42" s="4" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="H42" s="5" t="inlineStr"/>
+      <c r="I42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
@@ -34927,25 +35123,30 @@
       <c r="C43" s="5" t="inlineStr"/>
       <c r="D43" s="5" t="inlineStr">
         <is>
+          <t>作为犹他大学住宿与餐饮项目（HDP）的一线代表，为住户、访客和校内员工提供服务，同时协助住宿运营、宣传 HDP 资源并维…</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
           <t>住宿与居住教育</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
+      <c r="F43" s="4" t="inlineStr">
         <is>
           <t>19.99</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr">
+      <c r="G43" s="4" t="inlineStr">
         <is>
           <t>$14</t>
         </is>
       </c>
-      <c r="G43" s="4" t="inlineStr">
+      <c r="H43" s="4" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="H43" s="5" t="inlineStr"/>
+      <c r="I43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n">
@@ -34963,25 +35164,30 @@
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
+          <t>Prosperity U 招聘一名学生社交媒体实习生，每周最多工作 20 小时，负责各平台内容的管理、制作、互动和数据跟…</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
           <t>商业、健康与繁荣中心</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="F44" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F44" s="4" t="inlineStr">
+      <c r="G44" s="4" t="inlineStr">
         <is>
           <t>$14</t>
         </is>
       </c>
-      <c r="G44" s="4" t="inlineStr">
+      <c r="H44" s="4" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="H44" s="5" t="inlineStr"/>
+      <c r="I44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -34995,25 +35201,30 @@
       <c r="C45" s="5" t="inlineStr"/>
       <c r="D45" s="5" t="inlineStr">
         <is>
+          <t>代表建筑与规划学院（CA+P）接待意向学生、在校生、家长、校友和访客</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
           <t>建筑与规划学院</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
+      <c r="F45" s="4" t="inlineStr">
         <is>
           <t>8-12</t>
         </is>
       </c>
-      <c r="F45" s="4" t="inlineStr">
+      <c r="G45" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G45" s="4" t="inlineStr">
+      <c r="H45" s="4" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="H45" s="5" t="inlineStr"/>
+      <c r="I45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n">
@@ -35027,25 +35238,30 @@
       <c r="C46" s="5" t="inlineStr"/>
       <c r="D46" s="5" t="inlineStr">
         <is>
+          <t>协助 Red Butte Garden 露天剧场的户外音乐会和部分活动完成搭建、撤场和维护</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
           <t>Red Butte 植物园</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="F46" s="4" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="F46" s="4" t="inlineStr">
+      <c r="G46" s="4" t="inlineStr">
         <is>
           <t>$15.5</t>
         </is>
       </c>
-      <c r="G46" s="4" t="inlineStr">
+      <c r="H46" s="4" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="H46" s="5" t="inlineStr">
+      <c r="I46" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -35063,25 +35279,30 @@
       <c r="C47" s="5" t="inlineStr"/>
       <c r="D47" s="5" t="inlineStr">
         <is>
+          <t>David Eccles 商学院的 Professional MBA 和 Online MBA 项目招聘一名可靠、服务意…</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
           <t>高管教育</t>
         </is>
       </c>
-      <c r="E47" s="4" t="inlineStr">
+      <c r="F47" s="4" t="inlineStr">
         <is>
           <t>10–19 hours per week, with the potential for increased hours during the summer.</t>
         </is>
       </c>
-      <c r="F47" s="4" t="inlineStr">
+      <c r="G47" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G47" s="4" t="inlineStr">
+      <c r="H47" s="4" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="H47" s="5" t="inlineStr"/>
+      <c r="I47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n">
@@ -35095,25 +35316,30 @@
       <c r="C48" s="5" t="inlineStr"/>
       <c r="D48" s="5" t="inlineStr">
         <is>
+          <t>国际学生与学者服务办公室（ISSS）招聘一名友好、有同理心且积极的同伴助理，为犹他大学国际学生和学者提供支持</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
           <t>国际学生与学者服务中心</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="F48" s="4" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="F48" s="4" t="inlineStr">
+      <c r="G48" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G48" s="4" t="inlineStr">
+      <c r="H48" s="4" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="H48" s="5" t="inlineStr"/>
+      <c r="I48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n">
@@ -35131,25 +35357,30 @@
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
+          <t>加入较高级别的 IT 团队，协助管理 Apple、Microsoft 系统及其配套基础设施，为校园核心服务点的学生、教职…</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
           <t>Marriott 图书馆运营</t>
         </is>
       </c>
-      <c r="E49" s="4" t="inlineStr">
+      <c r="F49" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F49" s="4" t="inlineStr">
+      <c r="G49" s="4" t="inlineStr">
         <is>
           <t>$16</t>
         </is>
       </c>
-      <c r="G49" s="4" t="inlineStr">
+      <c r="H49" s="4" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="H49" s="5" t="inlineStr">
+      <c r="I49" s="5" t="inlineStr">
         <is>
           <t>需熟悉 Jamf Pro / SCCM，会脚本（Bash/PowerShell/Python/C/C++）</t>
         </is>
@@ -35171,25 +35402,30 @@
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
+          <t>University Analytics and Institutional Reporting（UAIR）招聘传播、市…</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
           <t>大学分析与机构报告</t>
         </is>
       </c>
-      <c r="E50" s="4" t="inlineStr">
+      <c r="F50" s="4" t="inlineStr">
         <is>
           <t>19 hours</t>
         </is>
       </c>
-      <c r="F50" s="4" t="inlineStr">
+      <c r="G50" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G50" s="4" t="inlineStr">
+      <c r="H50" s="4" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="H50" s="5" t="inlineStr"/>
+      <c r="I50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
@@ -35207,25 +35443,30 @@
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
+          <t>University Analytics and Institutional Reporting（UAIR）招聘计算机科…</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
           <t>大学分析与机构报告</t>
         </is>
       </c>
-      <c r="E51" s="4" t="inlineStr">
+      <c r="F51" s="4" t="inlineStr">
         <is>
           <t>19 hours per week</t>
         </is>
       </c>
-      <c r="F51" s="4" t="inlineStr">
+      <c r="G51" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G51" s="4" t="inlineStr">
+      <c r="H51" s="4" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="H51" s="5" t="inlineStr"/>
+      <c r="I51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="n">
@@ -35239,25 +35480,30 @@
       <c r="C52" s="5" t="inlineStr"/>
       <c r="D52" s="5" t="inlineStr">
         <is>
+          <t>在酒店前台值夜班，常规班次为 23:00 至次日 07:00，需要在节假日和周末工作，并可能按需要安排在一周中的任何一天</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
           <t>大学宾馆</t>
         </is>
       </c>
-      <c r="E52" s="4" t="inlineStr">
+      <c r="F52" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F52" s="4" t="inlineStr">
+      <c r="G52" s="4" t="inlineStr">
         <is>
           <t>$19</t>
         </is>
       </c>
-      <c r="G52" s="4" t="inlineStr">
+      <c r="H52" s="4" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="H52" s="5" t="inlineStr">
+      <c r="I52" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -35275,25 +35521,30 @@
       <c r="C53" s="5" t="inlineStr"/>
       <c r="D53" s="5" t="inlineStr">
         <is>
+          <t>完成各类清洁工作，维持清洁、卫生、无安全及感染隐患的环境，为员工、访客和患者提供安全整洁的空间</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
           <t>住宿与居住教育</t>
         </is>
       </c>
-      <c r="E53" s="4" t="inlineStr">
+      <c r="F53" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="F53" s="4" t="inlineStr">
+      <c r="G53" s="4" t="inlineStr">
         <is>
           <t>$16.16</t>
         </is>
       </c>
-      <c r="G53" s="4" t="inlineStr">
+      <c r="H53" s="4" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>
       </c>
-      <c r="H53" s="5" t="inlineStr"/>
+      <c r="I53" s="5" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n">
@@ -35311,25 +35562,30 @@
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
+          <t>在 Rice-Eccles Stadium 和 Jon M. Huntsman Center 的音乐会及特别活动中协助餐…</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
           <t>Rice-Eccles 体育场</t>
         </is>
       </c>
-      <c r="E54" s="4" t="inlineStr">
+      <c r="F54" s="4" t="inlineStr">
         <is>
           <t>10-15</t>
         </is>
       </c>
-      <c r="F54" s="4" t="inlineStr">
+      <c r="G54" s="4" t="inlineStr">
         <is>
           <t>$19</t>
         </is>
       </c>
-      <c r="G54" s="4" t="inlineStr">
+      <c r="H54" s="4" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="H54" s="5" t="inlineStr">
+      <c r="I54" s="5" t="inlineStr">
         <is>
           <t>年满 21 岁、需酒类服务证</t>
         </is>
@@ -35347,25 +35603,30 @@
       <c r="C55" s="5" t="inlineStr"/>
       <c r="D55" s="5" t="inlineStr">
         <is>
+          <t>可持续发展教育办公室招聘 SCIF 可持续发展大使，协助在犹他大学推广可持续发展教育</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
           <t>可持续校园倡议基金</t>
         </is>
       </c>
-      <c r="E55" s="4" t="inlineStr">
+      <c r="F55" s="4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="F55" s="4" t="inlineStr">
+      <c r="G55" s="4" t="inlineStr">
         <is>
           <t>$16</t>
         </is>
       </c>
-      <c r="G55" s="4" t="inlineStr">
+      <c r="H55" s="4" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="H55" s="5" t="inlineStr"/>
+      <c r="I55" s="5" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="n">
@@ -35379,25 +35640,30 @@
       <c r="C56" s="5" t="inlineStr"/>
       <c r="D56" s="5" t="inlineStr">
         <is>
+          <t>可持续发展教育办公室招聘实践学习可持续发展大使，协助在犹他大学推广可持续发展教育</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
           <t>可持续校园倡议基金</t>
         </is>
       </c>
-      <c r="E56" s="4" t="inlineStr">
+      <c r="F56" s="4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="F56" s="4" t="inlineStr">
+      <c r="G56" s="4" t="inlineStr">
         <is>
           <t>$16</t>
         </is>
       </c>
-      <c r="G56" s="4" t="inlineStr">
+      <c r="H56" s="4" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="H56" s="5" t="inlineStr"/>
+      <c r="I56" s="5" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n">
@@ -35411,25 +35677,30 @@
       <c r="C57" s="5" t="inlineStr"/>
       <c r="D57" s="5" t="inlineStr">
         <is>
+          <t>John and Marcia Price 工程学院电子与计算机工程系（ECE）招聘兼职行政助理，为院系工作及特定项目的…</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
           <t>电子与计算机工程系</t>
         </is>
       </c>
-      <c r="E57" s="4" t="inlineStr">
+      <c r="F57" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F57" s="4" t="inlineStr">
+      <c r="G57" s="4" t="inlineStr">
         <is>
           <t>$7.25</t>
         </is>
       </c>
-      <c r="G57" s="4" t="inlineStr">
+      <c r="H57" s="4" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="H57" s="5" t="inlineStr"/>
+      <c r="I57" s="5" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="n">
@@ -35447,25 +35718,30 @@
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
+          <t>保障大型体育和娱乐活动中的销售终端、数字标牌及合规设备正常运行</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
           <t>Rice-Eccles 体育场</t>
         </is>
       </c>
-      <c r="E58" s="4" t="inlineStr">
+      <c r="F58" s="4" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="F58" s="4" t="inlineStr">
+      <c r="G58" s="4" t="inlineStr">
         <is>
           <t>$16</t>
         </is>
       </c>
-      <c r="G58" s="4" t="inlineStr">
+      <c r="H58" s="4" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="H58" s="5" t="inlineStr">
+      <c r="I58" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -35487,25 +35763,30 @@
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
+          <t>在建筑与规划学院（CA+P）传播助理主任的指导下，负责面向在校生、意向学生、校友和社区合作伙伴开展传播工作</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
           <t>多学科设计系</t>
         </is>
       </c>
-      <c r="E59" s="4" t="inlineStr">
+      <c r="F59" s="4" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="F59" s="4" t="inlineStr">
+      <c r="G59" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G59" s="4" t="inlineStr">
+      <c r="H59" s="4" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="H59" s="5" t="inlineStr"/>
+      <c r="I59" s="5" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="n">
@@ -35523,25 +35804,30 @@
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
+          <t>STEM Community Alliance Program（STEMCAP）自 2016 年起，已在犹他州北部青少年…</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
           <t>本科生教育倡导项目</t>
         </is>
       </c>
-      <c r="E60" s="4" t="inlineStr">
+      <c r="F60" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F60" s="4" t="inlineStr">
+      <c r="G60" s="4" t="inlineStr">
         <is>
           <t>$25</t>
         </is>
       </c>
-      <c r="G60" s="4" t="inlineStr">
+      <c r="H60" s="4" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="H60" s="5" t="inlineStr">
+      <c r="I60" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -35563,25 +35849,30 @@
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
+          <t>承担音乐厅技术工作的部分或全部任务，包括后台舞台管理、灯光、音频、视频，以及与前厅团队协调；活动期间同时担任场馆代表</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
           <t>音乐学院</t>
         </is>
       </c>
-      <c r="E61" s="4" t="inlineStr">
+      <c r="F61" s="4" t="inlineStr">
         <is>
           <t>Varries based on performance/event schedule</t>
         </is>
       </c>
-      <c r="F61" s="4" t="inlineStr">
+      <c r="G61" s="4" t="inlineStr">
         <is>
           <t>$13</t>
         </is>
       </c>
-      <c r="G61" s="4" t="inlineStr">
+      <c r="H61" s="4" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="H61" s="5" t="inlineStr">
+      <c r="I61" s="5" t="inlineStr">
         <is>
           <t>需经验；需 2 年剧场舞台技术经验</t>
         </is>
@@ -35603,25 +35894,30 @@
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
+          <t>David Eccles 商学院招聘职业发展经理兼教练，为医疗管理硕士（MHA）学生提供职业支持，并参与项目的行业合作和…</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
           <t>高管教育</t>
         </is>
       </c>
-      <c r="E62" s="4" t="inlineStr">
+      <c r="F62" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F62" s="4" t="inlineStr">
+      <c r="G62" s="4" t="inlineStr">
         <is>
           <t>$30</t>
         </is>
       </c>
-      <c r="G62" s="4" t="inlineStr">
+      <c r="H62" s="4" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="H62" s="5" t="inlineStr">
+      <c r="I62" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -35643,25 +35939,30 @@
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
+          <t>协助犹他大学学生会开展学生项目和品牌宣传，负责印刷与数字营销活动、广告物料分发维护、社交媒体和网站内容发布，以及平面设计…</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
           <t>学生会</t>
         </is>
       </c>
-      <c r="E63" s="4" t="inlineStr">
+      <c r="F63" s="4" t="inlineStr">
         <is>
           <t>up to 19 hours/week</t>
         </is>
       </c>
-      <c r="F63" s="4" t="inlineStr">
+      <c r="G63" s="4" t="inlineStr">
         <is>
           <t>$14</t>
         </is>
       </c>
-      <c r="G63" s="4" t="inlineStr">
+      <c r="H63" s="4" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="H63" s="5" t="inlineStr"/>
+      <c r="I63" s="5" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="4" t="n">
@@ -35675,25 +35976,30 @@
       <c r="C64" s="5" t="inlineStr"/>
       <c r="D64" s="5" t="inlineStr">
         <is>
+          <t>犹他大学校园商店招聘一名可靠、细致的 Utech 技术服务助理</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
           <t>校园商店</t>
         </is>
       </c>
-      <c r="E64" s="4" t="inlineStr">
+      <c r="F64" s="4" t="inlineStr">
         <is>
           <t>19-20</t>
         </is>
       </c>
-      <c r="F64" s="4" t="inlineStr">
+      <c r="G64" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G64" s="4" t="inlineStr">
+      <c r="H64" s="4" t="inlineStr">
         <is>
           <t>2026-10-03</t>
         </is>
       </c>
-      <c r="H64" s="5" t="inlineStr">
+      <c r="I64" s="5" t="inlineStr">
         <is>
           <t>需通过安全审查（security clearance）</t>
         </is>
@@ -35711,25 +36017,30 @@
       <c r="C65" s="5" t="inlineStr"/>
       <c r="D65" s="5" t="inlineStr">
         <is>
+          <t>犹他大学校园商店招聘兼职订单履约助理，支持订单履约部门的日常运营</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
           <t>校园商店</t>
         </is>
       </c>
-      <c r="E65" s="4" t="inlineStr">
+      <c r="F65" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="F65" s="4" t="inlineStr">
+      <c r="G65" s="4" t="inlineStr">
         <is>
           <t>$14.5</t>
         </is>
       </c>
-      <c r="G65" s="4" t="inlineStr">
+      <c r="H65" s="4" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="H65" s="5" t="inlineStr"/>
+      <c r="I65" s="5" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="n">
@@ -35747,25 +36058,30 @@
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
+          <t>负责校内体育比赛的执裁和现场监督，执行竞赛规则，协助赛前器材布置与安全检查、赛后收尾、伤情应对和基础急救，并在冲突升级前…</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
           <t>校内体育</t>
         </is>
       </c>
-      <c r="E66" s="4" t="inlineStr">
+      <c r="F66" s="4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F66" s="4" t="inlineStr">
+      <c r="G66" s="4" t="inlineStr">
         <is>
           <t>$12</t>
         </is>
       </c>
-      <c r="G66" s="4" t="inlineStr">
+      <c r="H66" s="4" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>
       </c>
-      <c r="H66" s="5" t="inlineStr">
+      <c r="I66" s="5" t="inlineStr">
         <is>
           <t>需 CPR 认证（可入职一月内取得）</t>
         </is>
@@ -35783,25 +36099,30 @@
       <c r="C67" s="5" t="inlineStr"/>
       <c r="D67" s="5" t="inlineStr">
         <is>
+          <t>在 Rice-Eccles Stadium 和 Jon M. Huntsman Center 的活动中，根据仓库主管安排…</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
           <t>Rice-Eccles 体育场</t>
         </is>
       </c>
-      <c r="E67" s="4" t="inlineStr">
+      <c r="F67" s="4" t="inlineStr">
         <is>
           <t>4 hours per week or less</t>
         </is>
       </c>
-      <c r="F67" s="4" t="inlineStr">
+      <c r="G67" s="4" t="inlineStr">
         <is>
           <t>$16</t>
         </is>
       </c>
-      <c r="G67" s="4" t="inlineStr">
+      <c r="H67" s="4" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="H67" s="5" t="inlineStr">
+      <c r="I67" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -35819,25 +36140,30 @@
       <c r="C68" s="5" t="inlineStr"/>
       <c r="D68" s="5" t="inlineStr">
         <is>
+          <t>在体育场餐饮柜台准备和售卖三明治、沙拉、水果等食品，按标准控制份量并及时服务顾客；同时负责食品储存、工作区域与设备清洁消…</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
           <t>Rice-Eccles 体育场</t>
         </is>
       </c>
-      <c r="E68" s="4" t="inlineStr">
+      <c r="F68" s="4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F68" s="4" t="inlineStr">
+      <c r="G68" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G68" s="4" t="inlineStr">
+      <c r="H68" s="4" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="H68" s="5" t="inlineStr">
+      <c r="I68" s="5" t="inlineStr">
         <is>
           <t>需食品证</t>
         </is>
@@ -35855,25 +36181,30 @@
       <c r="C69" s="5" t="inlineStr"/>
       <c r="D69" s="5" t="inlineStr">
         <is>
+          <t>完成各类清洁工作，维持清洁、卫生、无安全及感染隐患的环境，为员工、访客和患者提供安全整洁的空间</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
           <t>住宿与居住教育</t>
         </is>
       </c>
-      <c r="E69" s="4" t="inlineStr">
+      <c r="F69" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F69" s="4" t="inlineStr">
+      <c r="G69" s="4" t="inlineStr">
         <is>
           <t>$16.16</t>
         </is>
       </c>
-      <c r="G69" s="4" t="inlineStr">
+      <c r="H69" s="4" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="H69" s="5" t="inlineStr"/>
+      <c r="I69" s="5" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="4" t="n">
@@ -35891,25 +36222,30 @@
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
+          <t>犹他美术博物馆（UMFA）位于犹他大学校园内，成立于 1914 年，是犹他州的官方美术博物馆</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
           <t>犹他美术博物馆</t>
         </is>
       </c>
-      <c r="E70" s="4" t="inlineStr">
+      <c r="F70" s="4" t="inlineStr">
         <is>
           <t>1-19</t>
         </is>
       </c>
-      <c r="F70" s="4" t="inlineStr">
+      <c r="G70" s="4" t="inlineStr">
         <is>
           <t>$14</t>
         </is>
       </c>
-      <c r="G70" s="4" t="inlineStr">
+      <c r="H70" s="4" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="H70" s="5" t="inlineStr">
+      <c r="I70" s="5" t="inlineStr">
         <is>
           <t>需食品证</t>
         </is>
@@ -35927,25 +36263,30 @@
       <c r="C71" s="5" t="inlineStr"/>
       <c r="D71" s="5" t="inlineStr">
         <is>
+          <t>犹他美术博物馆（UMFA）商店招聘一名积极、可靠、有创意的店员</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
           <t>犹他美术博物馆</t>
         </is>
       </c>
-      <c r="E71" s="4" t="inlineStr">
+      <c r="F71" s="4" t="inlineStr">
         <is>
           <t>1-19</t>
         </is>
       </c>
-      <c r="F71" s="4" t="inlineStr">
+      <c r="G71" s="4" t="inlineStr">
         <is>
           <t>$13.65</t>
         </is>
       </c>
-      <c r="G71" s="4" t="inlineStr">
+      <c r="H71" s="4" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="H71" s="5" t="inlineStr">
+      <c r="I71" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -35967,25 +36308,30 @@
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
+          <t>驾驶安保车辆</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
           <t>通勤服务</t>
         </is>
       </c>
-      <c r="E72" s="4" t="inlineStr">
+      <c r="F72" s="4" t="inlineStr">
         <is>
           <t>15-19 hours per week</t>
         </is>
       </c>
-      <c r="F72" s="4" t="inlineStr">
+      <c r="G72" s="4" t="inlineStr">
         <is>
           <t>$15.38</t>
         </is>
       </c>
-      <c r="G72" s="4" t="inlineStr">
+      <c r="H72" s="4" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="H72" s="5" t="inlineStr">
+      <c r="I72" s="5" t="inlineStr">
         <is>
           <t>需驾照</t>
         </is>
@@ -36003,25 +36349,30 @@
       <c r="C73" s="5" t="inlineStr"/>
       <c r="D73" s="5" t="inlineStr">
         <is>
+          <t>为继续教育部门提供数据录入、客户服务和基础教室技术支持，包括协助师生使用打印及影音设备、办理课程注册、巡查教室和维护物资</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
           <t>财务与运营</t>
         </is>
       </c>
-      <c r="E73" s="4" t="inlineStr">
+      <c r="F73" s="4" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="F73" s="4" t="inlineStr">
+      <c r="G73" s="4" t="inlineStr">
         <is>
           <t>$16</t>
         </is>
       </c>
-      <c r="G73" s="4" t="inlineStr">
+      <c r="H73" s="4" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="H73" s="5" t="inlineStr">
+      <c r="I73" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -36043,25 +36394,30 @@
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
+          <t>协助执行犹他美术博物馆（UMFA）的内部和外部活动，包括展览开幕式、筹款晚宴、会员活动、嘉宾讲座、婚礼和企业活动</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
           <t>犹他美术博物馆</t>
         </is>
       </c>
-      <c r="E74" s="4" t="inlineStr">
+      <c r="F74" s="4" t="inlineStr">
         <is>
           <t>0-19</t>
         </is>
       </c>
-      <c r="F74" s="4" t="inlineStr">
+      <c r="G74" s="4" t="inlineStr">
         <is>
           <t>$13.65</t>
         </is>
       </c>
-      <c r="G74" s="4" t="inlineStr">
+      <c r="H74" s="4" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H74" s="5" t="inlineStr">
+      <c r="I74" s="5" t="inlineStr">
         <is>
           <t>需经验；能提举 50 磅</t>
         </is>
@@ -36083,25 +36439,30 @@
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
+          <t>驾驶校园接驳班车</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
           <t>通勤服务</t>
         </is>
       </c>
-      <c r="E75" s="4" t="inlineStr">
+      <c r="F75" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="F75" s="4" t="inlineStr">
+      <c r="G75" s="4" t="inlineStr">
         <is>
           <t>$20</t>
         </is>
       </c>
-      <c r="G75" s="4" t="inlineStr">
+      <c r="H75" s="4" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="H75" s="5" t="inlineStr">
+      <c r="I75" s="5" t="inlineStr">
         <is>
           <t>需 CDL 驾照（提供付费培训）</t>
         </is>
@@ -36119,25 +36480,30 @@
       <c r="C76" s="5" t="inlineStr"/>
       <c r="D76" s="5" t="inlineStr">
         <is>
+          <t>完成各类清洁工作，维持清洁、卫生、无安全及感染隐患的环境，为员工、访客和患者提供安全整洁的空间</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
           <t>住宿与居住教育</t>
         </is>
       </c>
-      <c r="E76" s="4" t="inlineStr">
+      <c r="F76" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F76" s="4" t="inlineStr">
+      <c r="G76" s="4" t="inlineStr">
         <is>
           <t>$16.16</t>
         </is>
       </c>
-      <c r="G76" s="4" t="inlineStr">
+      <c r="H76" s="4" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="H76" s="5" t="inlineStr"/>
+      <c r="I76" s="5" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="n">
@@ -36155,25 +36521,30 @@
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
+          <t>为校园健康中心制作社交媒体、印刷品、演示文稿、网站和宣传活动所需的视觉内容，协助短视频、文案、内容排期及线上互动，并维护…</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
           <t>校园健康中心</t>
         </is>
       </c>
-      <c r="E77" s="4" t="inlineStr">
+      <c r="F77" s="4" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="F77" s="4" t="inlineStr">
+      <c r="G77" s="4" t="inlineStr">
         <is>
           <t>$14.5</t>
         </is>
       </c>
-      <c r="G77" s="4" t="inlineStr">
+      <c r="H77" s="4" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="H77" s="5" t="inlineStr"/>
+      <c r="I77" s="5" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="n">
@@ -36187,25 +36558,30 @@
       <c r="C78" s="5" t="inlineStr"/>
       <c r="D78" s="5" t="inlineStr">
         <is>
+          <t>协助 Academic Materials 部门的日常运营，为学生、教师和员工处理课程资料相关事务</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
           <t>校园商店</t>
         </is>
       </c>
-      <c r="E78" s="4" t="inlineStr">
+      <c r="F78" s="4" t="inlineStr">
         <is>
           <t>19-20</t>
         </is>
       </c>
-      <c r="F78" s="4" t="inlineStr">
+      <c r="G78" s="4" t="inlineStr">
         <is>
           <t>$14.5</t>
         </is>
       </c>
-      <c r="G78" s="4" t="inlineStr">
+      <c r="H78" s="4" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="H78" s="5" t="inlineStr"/>
+      <c r="I78" s="5" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="n">
@@ -36219,25 +36595,30 @@
       <c r="C79" s="5" t="inlineStr"/>
       <c r="D79" s="5" t="inlineStr">
         <is>
+          <t>犹他美术博物馆（UMFA）安保服务团队招聘一名积极、可靠的工作人员，在节奏较快、重视协作的环境中为团队提供支持</t>
+        </is>
+      </c>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
           <t>犹他美术博物馆</t>
         </is>
       </c>
-      <c r="E79" s="4" t="inlineStr">
+      <c r="F79" s="4" t="inlineStr">
         <is>
           <t>1-19</t>
         </is>
       </c>
-      <c r="F79" s="4" t="inlineStr">
+      <c r="G79" s="4" t="inlineStr">
         <is>
           <t>$13.65</t>
         </is>
       </c>
-      <c r="G79" s="4" t="inlineStr">
+      <c r="H79" s="4" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="H79" s="5" t="inlineStr">
+      <c r="I79" s="5" t="inlineStr">
         <is>
           <t>需驾照；需经验；需通过背景调查</t>
         </is>
@@ -36255,25 +36636,30 @@
       <c r="C80" s="5" t="inlineStr"/>
       <c r="D80" s="5" t="inlineStr">
         <is>
+          <t>Wilkes 气候科学与政策中心招聘一名学生大使，代表中心并帮助建立活跃的校园社区</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
           <t>Wilkes 气候科学与政策中心</t>
         </is>
       </c>
-      <c r="E80" s="4" t="inlineStr">
+      <c r="F80" s="4" t="inlineStr">
         <is>
           <t>10-15</t>
         </is>
       </c>
-      <c r="F80" s="4" t="inlineStr">
+      <c r="G80" s="4" t="inlineStr">
         <is>
           <t>$14</t>
         </is>
       </c>
-      <c r="G80" s="4" t="inlineStr">
+      <c r="H80" s="4" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="H80" s="5" t="inlineStr"/>
+      <c r="I80" s="5" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="n">
@@ -36287,25 +36673,30 @@
       <c r="C81" s="5" t="inlineStr"/>
       <c r="D81" s="5" t="inlineStr">
         <is>
+          <t>在首席研究员监督下完成实验技术操作</t>
+        </is>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
           <t>Huntsman 癌症研究所·Chandrasekharan 实验室</t>
         </is>
       </c>
-      <c r="E81" s="4" t="inlineStr">
+      <c r="F81" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="F81" s="4" t="inlineStr">
+      <c r="G81" s="4" t="inlineStr">
         <is>
           <t>$7.25</t>
         </is>
       </c>
-      <c r="G81" s="4" t="inlineStr">
+      <c r="H81" s="4" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="H81" s="5" t="inlineStr"/>
+      <c r="I81" s="5" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="n">
@@ -36319,25 +36710,30 @@
       <c r="C82" s="5" t="inlineStr"/>
       <c r="D82" s="5" t="inlineStr">
         <is>
+          <t>与他人共同管理餐饮售卖人员和验票志愿者，负责现金箱、库存、迟到观众入场安排、节目单装订与摆放，以及演出前和中场休息期间的…</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
           <t>先锋剧院</t>
         </is>
       </c>
-      <c r="E82" s="4" t="inlineStr">
+      <c r="F82" s="4" t="inlineStr">
         <is>
           <t>15-20</t>
         </is>
       </c>
-      <c r="F82" s="4" t="inlineStr">
+      <c r="G82" s="4" t="inlineStr">
         <is>
           <t>$11</t>
         </is>
       </c>
-      <c r="G82" s="4" t="inlineStr">
+      <c r="H82" s="4" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="H82" s="5" t="inlineStr">
+      <c r="I82" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -36355,25 +36751,30 @@
       <c r="C83" s="5" t="inlineStr"/>
       <c r="D83" s="5" t="inlineStr">
         <is>
+          <t>Pioneer Theatre Company 招聘票房收银员，负责接听电话、售票并回答顾客问题</t>
+        </is>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
           <t>先锋剧院</t>
         </is>
       </c>
-      <c r="E83" s="4" t="inlineStr">
+      <c r="F83" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="F83" s="4" t="inlineStr">
+      <c r="G83" s="4" t="inlineStr">
         <is>
           <t>$10.5</t>
         </is>
       </c>
-      <c r="G83" s="4" t="inlineStr">
+      <c r="H83" s="4" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="H83" s="5" t="inlineStr">
+      <c r="I83" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -36391,25 +36792,30 @@
       <c r="C84" s="5" t="inlineStr"/>
       <c r="D84" s="5" t="inlineStr">
         <is>
+          <t>提供常规办公室支持，审核并处理文件和信息申请，维护档案、录入数据并分发邮件</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
           <t>校园卡服务</t>
         </is>
       </c>
-      <c r="E84" s="4" t="inlineStr">
+      <c r="F84" s="4" t="inlineStr">
         <is>
           <t>15-19 hours per week</t>
         </is>
       </c>
-      <c r="F84" s="4" t="inlineStr">
+      <c r="G84" s="4" t="inlineStr">
         <is>
           <t>$15</t>
         </is>
       </c>
-      <c r="G84" s="4" t="inlineStr">
+      <c r="H84" s="4" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="H84" s="5" t="inlineStr">
+      <c r="I84" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -36431,25 +36837,30 @@
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
+          <t>UtahPresents 是犹他大学的非营利综合艺术演出机构，为校园及周边地区引进舞蹈、音乐会、喜剧、歌剧等项目</t>
+        </is>
+      </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
           <t>UtahPresents 演出项目</t>
         </is>
       </c>
-      <c r="E85" s="4" t="inlineStr">
+      <c r="F85" s="4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F85" s="4" t="inlineStr">
+      <c r="G85" s="4" t="inlineStr">
         <is>
           <t>$16</t>
         </is>
       </c>
-      <c r="G85" s="4" t="inlineStr">
+      <c r="H85" s="4" t="inlineStr">
         <is>
           <t>2026-11-05</t>
         </is>
       </c>
-      <c r="H85" s="5" t="inlineStr">
+      <c r="I85" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -36467,25 +36878,30 @@
       <c r="C86" s="5" t="inlineStr"/>
       <c r="D86" s="5" t="inlineStr">
         <is>
+          <t>为租用室内、室外网球场的顾客收款，办理预约和取消，接听场馆电话并处理顾客的问题，协助场馆经理完成其他前台事务</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
           <t>体育部</t>
         </is>
       </c>
-      <c r="E86" s="4" t="inlineStr">
+      <c r="F86" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F86" s="4" t="inlineStr">
+      <c r="G86" s="4" t="inlineStr">
         <is>
           <t>$7.25</t>
         </is>
       </c>
-      <c r="G86" s="4" t="inlineStr">
+      <c r="H86" s="4" t="inlineStr">
         <is>
           <t>2026-11-07</t>
         </is>
       </c>
-      <c r="H86" s="5" t="inlineStr"/>
+      <c r="I86" s="5" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="n">
@@ -36503,25 +36919,30 @@
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
+          <t>继续教育与社区参与部门下属的英语语言学院长期招聘线下面授 ESL 兼职教师</t>
+        </is>
+      </c>
+      <c r="E87" s="5" t="inlineStr">
+        <is>
           <t>英语语言学院</t>
         </is>
       </c>
-      <c r="E87" s="4" t="inlineStr">
+      <c r="F87" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F87" s="4" t="inlineStr">
+      <c r="G87" s="4" t="inlineStr">
         <is>
           <t>$49</t>
         </is>
       </c>
-      <c r="G87" s="4" t="inlineStr">
+      <c r="H87" s="4" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="H87" s="5" t="inlineStr">
+      <c r="I87" s="5" t="inlineStr">
         <is>
           <t>需 TESOL 硕士 + TESOL 证书</t>
         </is>
@@ -36539,25 +36960,30 @@
       <c r="C88" s="5" t="inlineStr"/>
       <c r="D88" s="5" t="inlineStr">
         <is>
+          <t>犹他大学 Impact &amp; Prosperity Epicenter 是一个以社会影响和共同繁荣为主题的住宿学习社区，通…</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
           <t>影响力与繁荣中心</t>
         </is>
       </c>
-      <c r="E88" s="4" t="inlineStr">
+      <c r="F88" s="4" t="inlineStr">
         <is>
           <t>15-19</t>
         </is>
       </c>
-      <c r="F88" s="4" t="inlineStr">
+      <c r="G88" s="4" t="inlineStr">
         <is>
           <t>$12</t>
         </is>
       </c>
-      <c r="G88" s="4" t="inlineStr">
+      <c r="H88" s="4" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="H88" s="5" t="inlineStr"/>
+      <c r="I88" s="5" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="n">
@@ -36575,25 +37001,30 @@
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
+          <t>在 Marriott Center for Dance 与视听室经理、技术总监、制作总监和舞台经理合作，负责舞蹈学院演出…</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
           <t>舞蹈学院</t>
         </is>
       </c>
-      <c r="E89" s="4" t="inlineStr">
+      <c r="F89" s="4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F89" s="4" t="inlineStr">
+      <c r="G89" s="4" t="inlineStr">
         <is>
           <t>$13.5</t>
         </is>
       </c>
-      <c r="G89" s="4" t="inlineStr">
+      <c r="H89" s="4" t="inlineStr">
         <is>
           <t>2026-12-31</t>
         </is>
       </c>
-      <c r="H89" s="5" t="inlineStr"/>
+      <c r="I89" s="5" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="n">
@@ -36611,31 +37042,36 @@
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
+          <t>在 Marriott Center for Dance 与制作总监、技术总监、舞台经理和视听室经理合作，为舞蹈学院演出及…</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
           <t>舞蹈学院</t>
         </is>
       </c>
-      <c r="E90" s="4" t="inlineStr">
+      <c r="F90" s="4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F90" s="4" t="inlineStr">
+      <c r="G90" s="4" t="inlineStr">
         <is>
           <t>$13.5</t>
         </is>
       </c>
-      <c r="G90" s="4" t="inlineStr">
+      <c r="H90" s="4" t="inlineStr">
         <is>
           <t>2026-12-31</t>
         </is>
       </c>
-      <c r="H90" s="5" t="inlineStr"/>
+      <c r="I90" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H90"/>
+  <autoFilter ref="A4:I90"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId1"/>

</xml_diff>

<commit_message>
Replace truncated summary with curated plain-language job descriptions, drop core-skills column
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'岗位检索'!$A$4:$W$126</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'MEAE国际学生省流版'!$A$4:$I$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'MEAE国际学生省流版'!$A$4:$H$90</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33421,18 +33421,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I90"/>
+  <dimension ref="A1:H90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -33463,35 +33462,30 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>核心能力</t>
+          <t>工作内容</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>工作内容</t>
+          <t>部门</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>部门</t>
+          <t>每周工时</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>每周工时</t>
+          <t>时薪</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>时薪</t>
+          <t>截止日期</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>截止日期</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>注意</t>
         </is>
@@ -33508,35 +33502,30 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>软件测试</t>
+          <t>软件测试、写测试脚本、自动化测试</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>在 University Information Technology（UIT）下属 University Suppor…</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
           <t>大学信息技术部·校级支持服务</t>
         </is>
       </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -33549,35 +33538,30 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>IT 技术支持</t>
+          <t>修电脑和 3D 打印机、巡视展项、处理工单</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>为现场和远程员工处理基础或一级 IT、视听问题，包括台式机、笔记本电脑和网络服务</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
           <t>犹他自然历史博物馆</t>
         </is>
       </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>$17</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>$17</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
           <t>2026-08-15</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -33594,35 +33578,30 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>统计分析、研究</t>
+          <t>迷幻药/心理健康研究：统计分析、写论文</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Yitong Xin 博士招聘一名研究生研究助理（职位代码 1632），支持团队不断增加的研究项目，主题包括迷幻药辅助治…</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
           <t>社会工作学院</t>
         </is>
       </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>未提供</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>未提供</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
           <t>2026-08-15</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>需社工硕士/博士在读，会 Mplus/SPSS/R</t>
         </is>
@@ -33639,35 +33618,30 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>人体模特</t>
+          <t>静坐摆姿势供艺术家绘画（着衣/裸体）</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>艺术与艺术史系招聘人体艺术模特，需要完成着衣和裸体姿势</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
           <t>艺术与艺术史系</t>
         </is>
       </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>0-6</t>
+        </is>
+      </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>0-6</t>
+          <t>$20</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>$20</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr"/>
+      <c r="H8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -33680,35 +33654,30 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>展品制作、手工</t>
+          <t>金属加工制作文物展示支架</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>为易损文物、标本和其他藏品设计、制作并安装符合文物保护要求的定制展示支架</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
           <t>犹他自然历史博物馆</t>
         </is>
       </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>$35</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>$35</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>需驾照；需经验</t>
         </is>
@@ -33725,35 +33694,30 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>社交媒体运营</t>
+          <t>给电台写社交帖、排期发布、拍短视频、监控互动</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>KUER 招聘一名有创意、注重细节的社交媒体助理，每周工作 19 小时，帮助扩大数字平台受众并提高互动</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
           <t>KUER 公共广播电台</t>
         </is>
       </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$17</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>$17</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -33768,33 +33732,32 @@
           <t>卖场助理</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr"/>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>商店轮岗：收银、理货、补货、接待</t>
+        </is>
+      </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>在校园商店多个业务区域轮岗，为顾客提供服务，并协助收银、商品陈列、补货和维护卖场</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
           <t>校园商店</t>
         </is>
       </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>19-20</t>
+        </is>
+      </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>19-20</t>
+          <t>DOE</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>DOE</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr"/>
+      <c r="H11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -33807,35 +33770,30 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>幼儿教育</t>
+          <t>带 0-6 岁幼儿、上课、照顾孩子</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Student Parent Support Center 为犹他大学学生、教职员工和患者提供信息、支持及家庭资源</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
           <t>学生家长支持中心</t>
         </is>
       </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$15.5</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>$15.5</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>食品证可后考；需经验；需 CPR/急救证，能抱举幼儿</t>
         </is>
@@ -33852,35 +33810,30 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>幼教辅助</t>
+          <t>协助幼教老师照顾孩子、组织活动</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Student Parent Support Center 为犹他大学学生、教职员工和患者提供信息、支持及家庭资源</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
           <t>学生家长支持中心</t>
         </is>
       </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>up to 19 hours/week, depending on hiring needs and incumbent schedule</t>
+        </is>
+      </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>up to 19 hours/week, depending on hiring needs and incumbent schedule</t>
+          <t>$14.5</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>$14.5</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>食品证可后考；入职 60 天内需食品证、TB 检测、BCI 背景调查、急救培训</t>
         </is>
@@ -33897,35 +33850,30 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>考试服务、技术支持</t>
+          <t>监考、帮师生用 Canvas、登记考生</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>面向大学生的入门岗位</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
           <t>在线教育</t>
         </is>
       </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$12</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>$12</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr"/>
+      <c r="H14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -33936,33 +33884,32 @@
           <t>收发货班次负责人</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr"/>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>管收发货物、验货、库存、带新人</t>
+        </is>
+      </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>犹他大学校园商店招聘兼职收发货班次文员，支持收发货部门的日常运营</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
           <t>校园商店</t>
         </is>
       </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>$16</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>$16</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -33979,35 +33926,30 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>韩语教学</t>
+          <t>教大一韩语课（KOREA 1010），改作业、出题</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>世界语言与文化系招聘兼职讲师，在 2026 年秋季学期教授一年级韩语</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
           <t>世界语言与文化系</t>
         </is>
       </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>4,200-6,000</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>4,200-6,000</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>需驾照；韩语接近母语级</t>
         </is>
@@ -34024,35 +33966,30 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>内容创作、营销</t>
+          <t>搜集整理校友内容、发简报和社交</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>在内容经理指导下协助校友传播和内容制作</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
           <t>校友关系办公室</t>
         </is>
       </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>8-10</t>
+        </is>
+      </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>8-10</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr"/>
+      <c r="H17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
@@ -34065,35 +34002,30 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>社交媒体运营</t>
+          <t>运营校友社交账号、活动拍照、整理内容</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>在主管 Emma 的指导下维护校友社交媒体账号，参与内容制作、活动报道和平台管理，重点做好故事表达、用户互动和内容组织</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
           <t>校友关系办公室</t>
         </is>
       </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr"/>
+      <c r="H18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -34104,33 +34036,32 @@
           <t>活动工作人员</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr"/>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>校友楼活动布置撤场、前台、引导</t>
+        </is>
+      </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Eccles Alumni House 招聘兼职活动工作人员，需要具备良好的顾客服务能力并能接受不固定排班</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
           <t>校友关系办公室</t>
         </is>
       </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>15-19</t>
+        </is>
+      </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>15-19</t>
+          <t>$15.6</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>$15.6</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr"/>
+      <c r="H19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
@@ -34143,35 +34074,30 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>市场调研</t>
+          <t>邮件营销、数据分析、A/B 测试（远程）</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>协助自然历史博物馆扩大 Research Quest 科学教育项目的全国影响力，主要负责自动化邮件营销、活动数据分析、A…</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
           <t>犹他自然历史博物馆</t>
         </is>
       </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>需经验；需本科学历+2年经验 或 硕士</t>
         </is>
@@ -34188,35 +34114,30 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>教学辅助</t>
+          <t>帮 MBA 老师做 Canvas 课程材料、批改、QA</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>为 MBA 项目教师提供支持，协助制作在线课程材料并进行质量检查，与教师、教学设计师和学生直接合作</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
           <t>高管教育</t>
         </is>
       </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>15 to 19</t>
+        </is>
+      </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>15 to 19</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="H21" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -34231,33 +34152,32 @@
           <t>楼宇服务助理</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr"/>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>图书馆设施维修维护：检查家具设备、小修、清洁、陪同承包商</t>
+        </is>
+      </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>负责 Marriott Library 的设施管理和维护，可独立完成分配的任务，也会与团队共同推进项目，并与不同部门合作…</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
           <t>Marriott 图书馆运营</t>
         </is>
       </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="I22" s="5" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>能提举 25 磅、爬梯凳</t>
         </is>
@@ -34272,33 +34192,32 @@
           <t>古生物藏品与登记助理</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr"/>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>录化石数据、扫描档案数字化</t>
+        </is>
+      </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>犹他自然历史博物馆招聘一名学生，协助古生物藏品管理和登记工作</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
           <t>犹他自然历史博物馆</t>
         </is>
       </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>$15.6</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>$15.6</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>需经验；需通过背景调查</t>
         </is>
@@ -34315,35 +34234,30 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>餐饮协调</t>
+          <t>管体育场餐饮摊位的员工培训和现场运营</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>负责监督犹他大学体育场和竞技馆餐饮服务，确保服务水平和操作标准持续达标；确认员工得到适当培训，并在需要时为他们提供现场协…</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
           <t>Rice-Eccles 体育场</t>
         </is>
       </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>16 hours per week or less</t>
+        </is>
+      </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>16 hours per week or less</t>
+          <t>$18</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>$18</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="I24" s="5" t="inlineStr">
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -34358,33 +34272,32 @@
           <t>设施维护助理</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr"/>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>体育场馆和草坪维护：割草、清洁、活动搭台</t>
+        </is>
+      </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>为体育设施、活动和运动草坪／场地运营提供一般支持，协助全职员工完成日常维护、活动搭建与撤场、设施保养，以及各体育场馆和户…</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
           <t>体育部</t>
         </is>
       </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$16</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>$16</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="I25" s="5" t="inlineStr">
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>需驾照；需经验；能提举 60 磅、需美国驾照</t>
         </is>
@@ -34401,35 +34314,30 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>摄影</t>
+          <t>在活动和周六服务项目里拍照、修图并上传</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>作为团队成员支持 Bennion Center for Community Engagement 的日常运营和各类项目需…</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
           <t>Bennion 社区参与中心</t>
         </is>
       </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>As needed</t>
+        </is>
+      </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>As needed</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I26" s="5" t="inlineStr"/>
+      <c r="H26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -34440,33 +34348,32 @@
           <t>成人教育项目助理</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr"/>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>协助花园的成人课程/讲座/工作坊，现场布置接待</t>
+        </is>
+      </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>加入 Red Butte Garden and Arboretum 成人项目部门，协助开展健康、创意、园艺、生态和烹饪等…</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
           <t>Red Butte 植物园</t>
         </is>
       </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$16</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>$16</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I27" s="5" t="inlineStr">
+      <c r="H27" s="5" t="inlineStr">
         <is>
           <t>需驾照；需经验；能提举 50 磅、走崎岖地形</t>
         </is>
@@ -34481,33 +34388,32 @@
           <t>现场服务办公室助理</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr"/>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>前台接待、接电话、文书、安排预约</t>
+        </is>
+      </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>当面或通过电话接待并协助访客，提供一般办公室支持</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
           <t>S.J. Quinney 法学院</t>
         </is>
       </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$9.62</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>$9.62</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I28" s="5" t="inlineStr">
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -34524,35 +34430,30 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>网络布线</t>
+          <t>铺网线/光纤、端接、按工单施工</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Pathway Engineering 团队负责建设和改善犹他大学物理网络层基础设施，包括在校园和医院楼宇内铺设、端接铜…</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
           <t>信息管理</t>
         </is>
       </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>15 - 19</t>
+        </is>
+      </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>15 - 19</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I29" s="5" t="inlineStr"/>
+      <c r="H29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
@@ -34565,35 +34466,30 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>活动策划</t>
+          <t>活动布置撤场、现场执行、后勤</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>商业、健康与繁荣中心位于 Impact &amp; Prosperity Epicenter，Prosperity U 是其面向…</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
           <t>商业、健康与繁荣中心</t>
         </is>
       </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>$12</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>$12</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I30" s="5" t="inlineStr"/>
+      <c r="H30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -34606,35 +34502,30 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Adobe 设计</t>
+          <t>教师生用 Adobe、办工作坊、技术支持</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>在 Kahlert Village 的 Adobe Creative Commons 担任创意软件顾问，帮助犹他大学师生…</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
           <t>大学信息技术部·数字学习技术</t>
         </is>
       </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H31" s="4" t="inlineStr">
-        <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I31" s="5" t="inlineStr">
+      <c r="H31" s="5" t="inlineStr">
         <is>
           <t>需精通至少 4 款 Adobe 应用</t>
         </is>
@@ -34651,35 +34542,30 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>媒体运营</t>
+          <t>管学生媒体的招聘、设备、市场和办公室</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>犹他大学 Student Media &amp; ABD 招聘学生担任办公室副经理</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
           <t>学生媒体委员会</t>
         </is>
       </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>15-20</t>
+        </is>
+      </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>15-20</t>
+          <t>$11</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>$11</t>
-        </is>
-      </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I32" s="5" t="inlineStr"/>
+      <c r="H32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -34690,33 +34576,32 @@
           <t>办公室助理</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr"/>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Nanofab 行政：接待、门禁、发票、库存</t>
+        </is>
+      </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Utah Nanofab 招聘一名办公室助理，为员工提供一般行政支持</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
           <t>犹他纳米制造实验室</t>
         </is>
       </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$7.25</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>$7.25</t>
-        </is>
-      </c>
-      <c r="H33" s="4" t="inlineStr">
-        <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I33" s="5" t="inlineStr"/>
+      <c r="H33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
@@ -34729,35 +34614,30 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>青少年项目</t>
+          <t>协助青少年气候行动项目、活动、评估</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>协助策划、执行和评估犹他自然历史博物馆 Critical Action Lab 项目的活动、会议和事件</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
           <t>犹他自然历史博物馆</t>
         </is>
       </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="I34" s="5" t="inlineStr">
+      <c r="H34" s="5" t="inlineStr">
         <is>
           <t>需驾照；需经验；需本科学历、驾照</t>
         </is>
@@ -34772,33 +34652,32 @@
           <t>酒店前台文员</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr"/>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>办入住退房、收银、接电话订房</t>
+        </is>
+      </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>接待酒店来宾，办理入住和退房，并协助处理问题或顾虑；有需要时也会在预订部门帮助客人订房，或支援早餐部门</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
           <t>大学宾馆</t>
         </is>
       </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="I35" s="5" t="inlineStr">
+      <c r="H35" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -34815,35 +34694,30 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>公众项目、教育</t>
+          <t>博物馆公众活动：协调志愿者、布置、协助</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>犹他自然历史博物馆（NHMU）的公众项目包括多种馆内活动，用于配合展览和馆藏，帮助访客了解自然世界并与社区建立联系</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
           <t>犹他自然历史博物馆</t>
         </is>
       </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H36" s="4" t="inlineStr">
-        <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="I36" s="5" t="inlineStr">
+      <c r="H36" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -34860,35 +34734,30 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>视频拍摄剪辑</t>
+          <t>给 MUSS/SAB 拍视频、剪辑、发社交</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>校友关系办公室招聘视频实习生，为 The Mighty Utah Student Section（MUSS）和 Stud…</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
           <t>校友关系办公室</t>
         </is>
       </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>15-19</t>
+        </is>
+      </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>15-19</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H37" s="4" t="inlineStr">
-        <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="I37" s="5" t="inlineStr">
+      <c r="H37" s="5" t="inlineStr">
         <is>
           <t>需会视频剪辑（Pr/达芬奇等）、DSLR/微单</t>
         </is>
@@ -34905,35 +34774,30 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>学位审核、数据处理</t>
+          <t>审核学生学位记录、核对课程、处理数据</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>为 Academic Progress 助理注册主任提供课程和学位审核方面的行政及分析支持，重点是通过学位审核确保学生学…</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
           <t>教务注册办公室</t>
         </is>
       </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>$20</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>$20</t>
-        </is>
-      </c>
-      <c r="H38" s="4" t="inlineStr">
-        <is>
           <t>2026-09-07</t>
         </is>
       </c>
-      <c r="I38" s="5" t="inlineStr">
+      <c r="H38" s="5" t="inlineStr">
         <is>
           <t>需经验；需本科学历 + 1 年相关经验</t>
         </is>
@@ -34950,35 +34814,30 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>停车执法</t>
+          <t>巡逻停车场、开违规罚单、指引停车</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>定期巡查并监督停车区域，处理违规停车，确保车位留给持有效许可的人员和特殊用途访客，同时为犹他大学师生和来访者提供服务</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
           <t>通勤服务</t>
         </is>
       </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$18</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>$18</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="inlineStr">
-        <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="I39" s="5" t="inlineStr">
+      <c r="H39" s="5" t="inlineStr">
         <is>
           <t>需驾照；需经验</t>
         </is>
@@ -34995,35 +34854,30 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>学业辅导</t>
+          <t>一对一辅导学生运动员，教时间管理和学习方法</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>为学生提供一对一或小组辅导，定期沟通以找出学习困难、改善学习方法并提高成绩</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
           <t>体育部</t>
         </is>
       </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$11</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>$11</t>
-        </is>
-      </c>
-      <c r="H40" s="4" t="inlineStr">
-        <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="I40" s="5" t="inlineStr">
+      <c r="H40" s="5" t="inlineStr">
         <is>
           <t>需经验；需通过 BCI 背景调查</t>
         </is>
@@ -35040,35 +34894,30 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>活动运营</t>
+          <t>体育赛事现场卖官方周边、运货、摆摊</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>支持犹他大学校园商店在橄榄球比赛、其他体育赛事和校内特别活动中销售官方授权的 Utah Athletics 服装、礼品和…</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
           <t>校园商店</t>
         </is>
       </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>$18</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>$18</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="inlineStr">
-        <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="I41" s="5" t="inlineStr">
+      <c r="H41" s="5" t="inlineStr">
         <is>
           <t>需驾照</t>
         </is>
@@ -35083,33 +34932,32 @@
           <t>招生办公室学生文员</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr"/>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>录入成绩单和申请、收发邮件、前台</t>
+        </is>
+      </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>招生办公室招聘学生文员，工作地点包括文件影像处理部门和本科招生材料处理部门</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
           <t>招生办公室</t>
         </is>
       </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>15-19 hours weekly</t>
+        </is>
+      </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>15-19 hours weekly</t>
+          <t>$14</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>$14</t>
-        </is>
-      </c>
-      <c r="H42" s="4" t="inlineStr">
-        <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="I42" s="5" t="inlineStr"/>
+      <c r="H42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
@@ -35120,33 +34968,32 @@
           <t>学生住宿大使</t>
         </is>
       </c>
-      <c r="C43" s="5" t="inlineStr"/>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>住宿前台接待、答住房问题、办入住退房</t>
+        </is>
+      </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>作为犹他大学住宿与餐饮项目（HDP）的一线代表，为住户、访客和校内员工提供服务，同时协助住宿运营、宣传 HDP 资源并维…</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
           <t>住宿与居住教育</t>
         </is>
       </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>19.99</t>
+        </is>
+      </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>19.99</t>
+          <t>$14</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>$14</t>
-        </is>
-      </c>
-      <c r="H43" s="4" t="inlineStr">
-        <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="I43" s="5" t="inlineStr"/>
+      <c r="H43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n">
@@ -35159,35 +35006,30 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>社交媒体运营</t>
+          <t>运营社交账号、拍活动、写帖子</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Prosperity U 招聘一名学生社交媒体实习生，每周最多工作 20 小时，负责各平台内容的管理、制作、互动和数据跟…</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
           <t>商业、健康与繁荣中心</t>
         </is>
       </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$14</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>$14</t>
-        </is>
-      </c>
-      <c r="H44" s="4" t="inlineStr">
-        <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="I44" s="5" t="inlineStr"/>
+      <c r="H44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -35198,33 +35040,32 @@
           <t>建筑与规划学院学生大使</t>
         </is>
       </c>
-      <c r="C45" s="5" t="inlineStr"/>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>带校园参观、招生活动、介绍学院</t>
+        </is>
+      </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>代表建筑与规划学院（CA+P）接待意向学生、在校生、家长、校友和访客</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
           <t>建筑与规划学院</t>
         </is>
       </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>8-12</t>
+        </is>
+      </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>8-12</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H45" s="4" t="inlineStr">
-        <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="I45" s="5" t="inlineStr"/>
+      <c r="H45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n">
@@ -35235,33 +35076,32 @@
           <t>活动支持专员</t>
         </is>
       </c>
-      <c r="C46" s="5" t="inlineStr"/>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>露天音乐会搭台撤场、搬物资、维持现场</t>
+        </is>
+      </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>协助 Red Butte Garden 露天剧场的户外音乐会和部分活动完成搭建、撤场和维护</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
           <t>Red Butte 植物园</t>
         </is>
       </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>$15.5</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>$15.5</t>
-        </is>
-      </c>
-      <c r="H46" s="4" t="inlineStr">
-        <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="I46" s="5" t="inlineStr">
+      <c r="H46" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -35276,33 +35116,32 @@
           <t>办公室与课堂支持助理</t>
         </is>
       </c>
-      <c r="C47" s="5" t="inlineStr"/>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>MBA 项目行政、活动支持、课堂技术</t>
+        </is>
+      </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>David Eccles 商学院的 Professional MBA 和 Online MBA 项目招聘一名可靠、服务意…</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
           <t>高管教育</t>
         </is>
       </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>10–19 hours per week, with the potential for increased hours during the summer.</t>
+        </is>
+      </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>10–19 hours per week, with the potential for increased hours during the summer.</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H47" s="4" t="inlineStr">
-        <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="I47" s="5" t="inlineStr"/>
+      <c r="H47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n">
@@ -35313,33 +35152,32 @@
           <t>国际学生与学者服务同伴助理</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr"/>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>ISSS 前台接待登记、答邮件电话</t>
+        </is>
+      </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>国际学生与学者服务办公室（ISSS）招聘一名友好、有同理心且积极的同伴助理，为犹他大学国际学生和学者提供支持</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
           <t>国际学生与学者服务中心</t>
         </is>
       </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H48" s="4" t="inlineStr">
-        <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="I48" s="5" t="inlineStr"/>
+      <c r="H48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n">
@@ -35352,35 +35190,30 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>系统管理、脚本</t>
+          <t>帮师生修电脑和系统问题、装软件、处理工单</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>加入较高级别的 IT 团队，协助管理 Apple、Microsoft 系统及其配套基础设施，为校园核心服务点的学生、教职…</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
           <t>Marriott 图书馆运营</t>
         </is>
       </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$16</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>$16</t>
-        </is>
-      </c>
-      <c r="H49" s="4" t="inlineStr">
-        <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="I49" s="5" t="inlineStr">
+      <c r="H49" s="5" t="inlineStr">
         <is>
           <t>需熟悉 Jamf Pro / SCCM，会脚本（Bash/PowerShell/Python/C/C++）</t>
         </is>
@@ -35397,35 +35230,30 @@
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>数据治理、传播</t>
+          <t>做数据治理培训材料、视频、网页内容</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>University Analytics and Institutional Reporting（UAIR）招聘传播、市…</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
           <t>大学分析与机构报告</t>
         </is>
       </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>19 hours</t>
+        </is>
+      </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>19 hours</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H50" s="4" t="inlineStr">
-        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="I50" s="5" t="inlineStr"/>
+      <c r="H50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
@@ -35438,35 +35266,30 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>数据治理、技术</t>
+          <t>写代码采集整合数据、做自动化 ETL</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>University Analytics and Institutional Reporting（UAIR）招聘计算机科…</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
           <t>大学分析与机构报告</t>
         </is>
       </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>19 hours per week</t>
+        </is>
+      </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>19 hours per week</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H51" s="4" t="inlineStr">
-        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="I51" s="5" t="inlineStr"/>
+      <c r="H51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="n">
@@ -35477,33 +35300,32 @@
           <t>酒店夜班前台文员</t>
         </is>
       </c>
-      <c r="C52" s="5" t="inlineStr"/>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>酒店夜班前台：办入住、跑审计、做存款</t>
+        </is>
+      </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>在酒店前台值夜班，常规班次为 23:00 至次日 07:00，需要在节假日和周末工作，并可能按需要安排在一周中的任何一天</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
           <t>大学宾馆</t>
         </is>
       </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$19</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
-          <t>$19</t>
-        </is>
-      </c>
-      <c r="H52" s="4" t="inlineStr">
-        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="I52" s="5" t="inlineStr">
+      <c r="H52" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -35518,33 +35340,32 @@
           <t>兼职保洁员</t>
         </is>
       </c>
-      <c r="C53" s="5" t="inlineStr"/>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>扫地拖地、清洁厕所、倒垃圾、维护地面</t>
+        </is>
+      </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>完成各类清洁工作，维持清洁、卫生、无安全及感染隐患的环境，为员工、访客和患者提供安全整洁的空间</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
           <t>住宿与居住教育</t>
         </is>
       </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>$16.16</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>$16.16</t>
-        </is>
-      </c>
-      <c r="H53" s="4" t="inlineStr">
-        <is>
           <t>2026-09-29</t>
         </is>
       </c>
-      <c r="I53" s="5" t="inlineStr"/>
+      <c r="H53" s="5" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n">
@@ -35557,35 +35378,30 @@
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>酒水服务</t>
+          <t>在体育馆卖酒水、查年龄、收银</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>在 Rice-Eccles Stadium 和 Jon M. Huntsman Center 的音乐会及特别活动中协助餐…</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
           <t>Rice-Eccles 体育场</t>
         </is>
       </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>$19</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>$19</t>
-        </is>
-      </c>
-      <c r="H54" s="4" t="inlineStr">
-        <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="I54" s="5" t="inlineStr">
+      <c r="H54" s="5" t="inlineStr">
         <is>
           <t>年满 21 岁、需酒类服务证</t>
         </is>
@@ -35600,33 +35416,32 @@
           <t>SCIF 可持续发展大使</t>
         </is>
       </c>
-      <c r="C55" s="5" t="inlineStr"/>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>协助可持续发展项目、摆摊外联、写宣传内容</t>
+        </is>
+      </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>可持续发展教育办公室招聘 SCIF 可持续发展大使，协助在犹他大学推广可持续发展教育</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
           <t>可持续校园倡议基金</t>
         </is>
       </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>$16</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>$16</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="I55" s="5" t="inlineStr"/>
+      <c r="H55" s="5" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="n">
@@ -35637,33 +35452,32 @@
           <t>实践学习可持续发展大使</t>
         </is>
       </c>
-      <c r="C56" s="5" t="inlineStr"/>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>协助可持续发展课程和项目、摆摊外联、写宣传</t>
+        </is>
+      </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>可持续发展教育办公室招聘实践学习可持续发展大使，协助在犹他大学推广可持续发展教育</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
           <t>可持续校园倡议基金</t>
         </is>
       </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>$16</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>$16</t>
-        </is>
-      </c>
-      <c r="H56" s="4" t="inlineStr">
-        <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="I56" s="5" t="inlineStr"/>
+      <c r="H56" s="5" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n">
@@ -35674,33 +35488,32 @@
           <t>电子与计算机工程系行政助理</t>
         </is>
       </c>
-      <c r="C57" s="5" t="inlineStr"/>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>系里前台、接电话、文书、数据录入</t>
+        </is>
+      </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>John and Marcia Price 工程学院电子与计算机工程系（ECE）招聘兼职行政助理，为院系工作及特定项目的…</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
           <t>电子与计算机工程系</t>
         </is>
       </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$7.25</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>$7.25</t>
-        </is>
-      </c>
-      <c r="H57" s="4" t="inlineStr">
-        <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="I57" s="5" t="inlineStr"/>
+      <c r="H57" s="5" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="n">
@@ -35713,35 +35526,30 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>餐饮技术</t>
+          <t>维护活动中的 POS 收款机、网络和数字标牌</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>保障大型体育和娱乐活动中的销售终端、数字标牌及合规设备正常运行</t>
-        </is>
-      </c>
-      <c r="E58" s="5" t="inlineStr">
-        <is>
           <t>Rice-Eccles 体育场</t>
         </is>
       </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>$16</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>$16</t>
-        </is>
-      </c>
-      <c r="H58" s="4" t="inlineStr">
-        <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="I58" s="5" t="inlineStr">
+      <c r="H58" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -35758,35 +35566,30 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>社交媒体运营</t>
+          <t>建筑学院社交媒体：写内容、拍活动、剪短视频</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>在建筑与规划学院（CA+P）传播助理主任的指导下，负责面向在校生、意向学生、校友和社区合作伙伴开展传播工作</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
           <t>多学科设计系</t>
         </is>
       </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H59" s="4" t="inlineStr">
-        <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="I59" s="5" t="inlineStr"/>
+      <c r="H59" s="5" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="n">
@@ -35799,35 +35602,30 @@
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>项目支持</t>
+          <t>在青少年中心办科学/艺术工作坊、主持活动</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>STEM Community Alliance Program（STEMCAP）自 2016 年起，已在犹他州北部青少年…</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
           <t>本科生教育倡导项目</t>
         </is>
       </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$25</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>$25</t>
-        </is>
-      </c>
-      <c r="H60" s="4" t="inlineStr">
-        <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="I60" s="5" t="inlineStr">
+      <c r="H60" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -35844,35 +35642,30 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>舞台管理</t>
+          <t>音乐厅舞台管理：灯光、音响、视频、布场</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>承担音乐厅技术工作的部分或全部任务，包括后台舞台管理、灯光、音频、视频，以及与前厅团队协调；活动期间同时担任场馆代表</t>
-        </is>
-      </c>
-      <c r="E61" s="5" t="inlineStr">
-        <is>
           <t>音乐学院</t>
         </is>
       </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>Varries based on performance/event schedule</t>
+        </is>
+      </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>Varries based on performance/event schedule</t>
+          <t>$13</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>$13</t>
-        </is>
-      </c>
-      <c r="H61" s="4" t="inlineStr">
-        <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="I61" s="5" t="inlineStr">
+      <c r="H61" s="5" t="inlineStr">
         <is>
           <t>需经验；需 2 年剧场舞台技术经验</t>
         </is>
@@ -35889,35 +35682,30 @@
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>职业咨询</t>
+          <t>给医疗管理硕士做职业辅导、雇主关系</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>David Eccles 商学院招聘职业发展经理兼教练，为医疗管理硕士（MHA）学生提供职业支持，并参与项目的行业合作和…</t>
-        </is>
-      </c>
-      <c r="E62" s="5" t="inlineStr">
-        <is>
           <t>高管教育</t>
         </is>
       </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$30</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>$30</t>
-        </is>
-      </c>
-      <c r="H62" s="4" t="inlineStr">
-        <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="I62" s="5" t="inlineStr">
+      <c r="H62" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -35934,35 +35722,30 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>市场营销、设计</t>
+          <t>学生会营销：做图、发社交媒体、摄影视频</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>协助犹他大学学生会开展学生项目和品牌宣传，负责印刷与数字营销活动、广告物料分发维护、社交媒体和网站内容发布，以及平面设计…</t>
-        </is>
-      </c>
-      <c r="E63" s="5" t="inlineStr">
-        <is>
           <t>学生会</t>
         </is>
       </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>up to 19 hours/week</t>
+        </is>
+      </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>up to 19 hours/week</t>
+          <t>$14</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>$14</t>
-        </is>
-      </c>
-      <c r="H63" s="4" t="inlineStr">
-        <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="I63" s="5" t="inlineStr"/>
+      <c r="H63" s="5" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="4" t="n">
@@ -35973,33 +35756,32 @@
           <t>Utech 技术服务助理</t>
         </is>
       </c>
-      <c r="C64" s="5" t="inlineStr"/>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>校园商店电脑维修、故障排查、接待顾客</t>
+        </is>
+      </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>犹他大学校园商店招聘一名可靠、细致的 Utech 技术服务助理</t>
-        </is>
-      </c>
-      <c r="E64" s="5" t="inlineStr">
-        <is>
           <t>校园商店</t>
         </is>
       </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>19-20</t>
+        </is>
+      </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>19-20</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H64" s="4" t="inlineStr">
-        <is>
           <t>2026-10-03</t>
         </is>
       </c>
-      <c r="I64" s="5" t="inlineStr">
+      <c r="H64" s="5" t="inlineStr">
         <is>
           <t>需通过安全审查（security clearance）</t>
         </is>
@@ -36014,33 +35796,32 @@
           <t>订单履约助理</t>
         </is>
       </c>
-      <c r="C65" s="5" t="inlineStr"/>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>拣货、包装、寄送线上订单</t>
+        </is>
+      </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>犹他大学校园商店招聘兼职订单履约助理，支持订单履约部门的日常运营</t>
-        </is>
-      </c>
-      <c r="E65" s="5" t="inlineStr">
-        <is>
           <t>校园商店</t>
         </is>
       </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>$14.5</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>$14.5</t>
-        </is>
-      </c>
-      <c r="H65" s="4" t="inlineStr">
-        <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="I65" s="5" t="inlineStr"/>
+      <c r="H65" s="5" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="n">
@@ -36053,35 +35834,30 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>体育裁判</t>
+          <t>执裁校内比赛、布置器材、做急救</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>负责校内体育比赛的执裁和现场监督，执行竞赛规则，协助赛前器材布置与安全检查、赛后收尾、伤情应对和基础急救，并在冲突升级前…</t>
-        </is>
-      </c>
-      <c r="E66" s="5" t="inlineStr">
-        <is>
           <t>校内体育</t>
         </is>
       </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>$12</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>$12</t>
-        </is>
-      </c>
-      <c r="H66" s="4" t="inlineStr">
-        <is>
           <t>2026-10-08</t>
         </is>
       </c>
-      <c r="I66" s="5" t="inlineStr">
+      <c r="H66" s="5" t="inlineStr">
         <is>
           <t>需 CPR 认证（可入职一月内取得）</t>
         </is>
@@ -36096,33 +35872,32 @@
           <t>仓库工作人员</t>
         </is>
       </c>
-      <c r="C67" s="5" t="inlineStr"/>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>体育馆活动期间搬货、补货、管仓库</t>
+        </is>
+      </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>在 Rice-Eccles Stadium 和 Jon M. Huntsman Center 的活动中，根据仓库主管安排…</t>
-        </is>
-      </c>
-      <c r="E67" s="5" t="inlineStr">
-        <is>
           <t>Rice-Eccles 体育场</t>
         </is>
       </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>4 hours per week or less</t>
+        </is>
+      </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>4 hours per week or less</t>
+          <t>$16</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>$16</t>
-        </is>
-      </c>
-      <c r="H67" s="4" t="inlineStr">
-        <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="I67" s="5" t="inlineStr">
+      <c r="H67" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -36137,33 +35912,32 @@
           <t>体育场餐饮售卖人员</t>
         </is>
       </c>
-      <c r="C68" s="5" t="inlineStr"/>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>在餐饮柜台做三明治/沙拉、卖餐、清洁消毒</t>
+        </is>
+      </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>在体育场餐饮柜台准备和售卖三明治、沙拉、水果等食品，按标准控制份量并及时服务顾客；同时负责食品储存、工作区域与设备清洁消…</t>
-        </is>
-      </c>
-      <c r="E68" s="5" t="inlineStr">
-        <is>
           <t>Rice-Eccles 体育场</t>
         </is>
       </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H68" s="4" t="inlineStr">
-        <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="I68" s="5" t="inlineStr">
+      <c r="H68" s="5" t="inlineStr">
         <is>
           <t>需食品证</t>
         </is>
@@ -36178,33 +35952,32 @@
           <t>兼职保洁员</t>
         </is>
       </c>
-      <c r="C69" s="5" t="inlineStr"/>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>扫地拖地、清洁厕所、倒垃圾、维护地面</t>
+        </is>
+      </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>完成各类清洁工作，维持清洁、卫生、无安全及感染隐患的环境，为员工、访客和患者提供安全整洁的空间</t>
-        </is>
-      </c>
-      <c r="E69" s="5" t="inlineStr">
-        <is>
           <t>住宿与居住教育</t>
         </is>
       </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$16.16</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>$16.16</t>
-        </is>
-      </c>
-      <c r="H69" s="4" t="inlineStr">
-        <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="I69" s="5" t="inlineStr"/>
+      <c r="H69" s="5" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="4" t="n">
@@ -36217,35 +35990,30 @@
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>后厨</t>
+          <t>后厨做餐、洗碗、清洁、备料</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>犹他美术博物馆（UMFA）位于犹他大学校园内，成立于 1914 年，是犹他州的官方美术博物馆</t>
-        </is>
-      </c>
-      <c r="E70" s="5" t="inlineStr">
-        <is>
           <t>犹他美术博物馆</t>
         </is>
       </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>1-19</t>
+        </is>
+      </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>1-19</t>
+          <t>$14</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>$14</t>
-        </is>
-      </c>
-      <c r="H70" s="4" t="inlineStr">
-        <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="I70" s="5" t="inlineStr">
+      <c r="H70" s="5" t="inlineStr">
         <is>
           <t>需食品证</t>
         </is>
@@ -36260,33 +36028,32 @@
           <t>UMFA 商店店员</t>
         </is>
       </c>
-      <c r="C71" s="5" t="inlineStr"/>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>博物馆商店接待顾客、收银、补货</t>
+        </is>
+      </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>犹他美术博物馆（UMFA）商店招聘一名积极、可靠、有创意的店员</t>
-        </is>
-      </c>
-      <c r="E71" s="5" t="inlineStr">
-        <is>
           <t>犹他美术博物馆</t>
         </is>
       </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>1-19</t>
+        </is>
+      </c>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>1-19</t>
+          <t>$13.65</t>
         </is>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>$13.65</t>
-        </is>
-      </c>
-      <c r="H71" s="4" t="inlineStr">
-        <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="I71" s="5" t="inlineStr">
+      <c r="H71" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -36303,35 +36070,30 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>驾驶、安保</t>
+          <t>开安保客货车随叫随到、车辆检查</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>驾驶安保车辆</t>
-        </is>
-      </c>
-      <c r="E72" s="5" t="inlineStr">
-        <is>
           <t>通勤服务</t>
         </is>
       </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>15-19 hours per week</t>
+        </is>
+      </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>15-19 hours per week</t>
+          <t>$15.38</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>$15.38</t>
-        </is>
-      </c>
-      <c r="H72" s="4" t="inlineStr">
-        <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="I72" s="5" t="inlineStr">
+      <c r="H72" s="5" t="inlineStr">
         <is>
           <t>需驾照</t>
         </is>
@@ -36346,33 +36108,32 @@
           <t>顾客服务代表</t>
         </is>
       </c>
-      <c r="C73" s="5" t="inlineStr"/>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>继续教育部：数据录入、客服、教室设备支持</t>
+        </is>
+      </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>为继续教育部门提供数据录入、客户服务和基础教室技术支持，包括协助师生使用打印及影音设备、办理课程注册、巡查教室和维护物资</t>
-        </is>
-      </c>
-      <c r="E73" s="5" t="inlineStr">
-        <is>
           <t>财务与运营</t>
         </is>
       </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>$16</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>$16</t>
-        </is>
-      </c>
-      <c r="H73" s="4" t="inlineStr">
-        <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="I73" s="5" t="inlineStr">
+      <c r="H73" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -36389,35 +36150,30 @@
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>活动支持</t>
+          <t>博物馆活动布置撤场、音视频、接待</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>协助执行犹他美术博物馆（UMFA）的内部和外部活动，包括展览开幕式、筹款晚宴、会员活动、嘉宾讲座、婚礼和企业活动</t>
-        </is>
-      </c>
-      <c r="E74" s="5" t="inlineStr">
-        <is>
           <t>犹他美术博物馆</t>
         </is>
       </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>0-19</t>
+        </is>
+      </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>0-19</t>
+          <t>$13.65</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>$13.65</t>
-        </is>
-      </c>
-      <c r="H74" s="4" t="inlineStr">
-        <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="I74" s="5" t="inlineStr">
+      <c r="H74" s="5" t="inlineStr">
         <is>
           <t>需经验；能提举 50 磅</t>
         </is>
@@ -36434,35 +36190,30 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>驾驶</t>
+          <t>开穿梭巴士接送学生、检查车辆</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>驾驶校园接驳班车</t>
-        </is>
-      </c>
-      <c r="E75" s="5" t="inlineStr">
-        <is>
           <t>通勤服务</t>
         </is>
       </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>$20</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>$20</t>
-        </is>
-      </c>
-      <c r="H75" s="4" t="inlineStr">
-        <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="I75" s="5" t="inlineStr">
+      <c r="H75" s="5" t="inlineStr">
         <is>
           <t>需 CDL 驾照（提供付费培训）</t>
         </is>
@@ -36477,33 +36228,32 @@
           <t>兼职保洁员</t>
         </is>
       </c>
-      <c r="C76" s="5" t="inlineStr"/>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>扫地拖地、清洁厕所、倒垃圾、维护地面</t>
+        </is>
+      </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>完成各类清洁工作，维持清洁、卫生、无安全及感染隐患的环境，为员工、访客和患者提供安全整洁的空间</t>
-        </is>
-      </c>
-      <c r="E76" s="5" t="inlineStr">
-        <is>
           <t>住宿与居住教育</t>
         </is>
       </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$16.16</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>$16.16</t>
-        </is>
-      </c>
-      <c r="H76" s="4" t="inlineStr">
-        <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="I76" s="5" t="inlineStr"/>
+      <c r="H76" s="5" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="n">
@@ -36516,35 +36266,30 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>市场营销</t>
+          <t>健康中心做图、短视频、发社交</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>为校园健康中心制作社交媒体、印刷品、演示文稿、网站和宣传活动所需的视觉内容，协助短视频、文案、内容排期及线上互动，并维护…</t>
-        </is>
-      </c>
-      <c r="E77" s="5" t="inlineStr">
-        <is>
           <t>校园健康中心</t>
         </is>
       </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>$14.5</t>
         </is>
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>$14.5</t>
-        </is>
-      </c>
-      <c r="H77" s="4" t="inlineStr">
-        <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="I77" s="5" t="inlineStr"/>
+      <c r="H77" s="5" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="n">
@@ -36555,33 +36300,32 @@
           <t>教材与课程资料助理</t>
         </is>
       </c>
-      <c r="C78" s="5" t="inlineStr"/>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>录教材数据、帮师生找教材、联系供应商</t>
+        </is>
+      </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>协助 Academic Materials 部门的日常运营，为学生、教师和员工处理课程资料相关事务</t>
-        </is>
-      </c>
-      <c r="E78" s="5" t="inlineStr">
-        <is>
           <t>校园商店</t>
         </is>
       </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>19-20</t>
+        </is>
+      </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>19-20</t>
+          <t>$14.5</t>
         </is>
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>$14.5</t>
-        </is>
-      </c>
-      <c r="H78" s="4" t="inlineStr">
-        <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="I78" s="5" t="inlineStr"/>
+      <c r="H78" s="5" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="n">
@@ -36592,33 +36336,32 @@
           <t>UMFA 安保服务人员</t>
         </is>
       </c>
-      <c r="C79" s="5" t="inlineStr"/>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>巡逻、监控、保护藏品、维持秩序</t>
+        </is>
+      </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>犹他美术博物馆（UMFA）安保服务团队招聘一名积极、可靠的工作人员，在节奏较快、重视协作的环境中为团队提供支持</t>
-        </is>
-      </c>
-      <c r="E79" s="5" t="inlineStr">
-        <is>
           <t>犹他美术博物馆</t>
         </is>
       </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>1-19</t>
+        </is>
+      </c>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>1-19</t>
+          <t>$13.65</t>
         </is>
       </c>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>$13.65</t>
-        </is>
-      </c>
-      <c r="H79" s="4" t="inlineStr">
-        <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="I79" s="5" t="inlineStr">
+      <c r="H79" s="5" t="inlineStr">
         <is>
           <t>需驾照；需经验；需通过背景调查</t>
         </is>
@@ -36633,33 +36376,32 @@
           <t>Wilkes 中心学生大使</t>
         </is>
       </c>
-      <c r="C80" s="5" t="inlineStr"/>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>代表气候中心做外联、摆摊、接待访客</t>
+        </is>
+      </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>Wilkes 气候科学与政策中心招聘一名学生大使，代表中心并帮助建立活跃的校园社区</t>
-        </is>
-      </c>
-      <c r="E80" s="5" t="inlineStr">
-        <is>
           <t>Wilkes 气候科学与政策中心</t>
         </is>
       </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>$14</t>
         </is>
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>$14</t>
-        </is>
-      </c>
-      <c r="H80" s="4" t="inlineStr">
-        <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="I80" s="5" t="inlineStr"/>
+      <c r="H80" s="5" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="n">
@@ -36670,33 +36412,32 @@
           <t>实验室助理</t>
         </is>
       </c>
-      <c r="C81" s="5" t="inlineStr"/>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>在实验室做细胞/分子生物学实验、配培养基、管耗材</t>
+        </is>
+      </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>在首席研究员监督下完成实验技术操作</t>
-        </is>
-      </c>
-      <c r="E81" s="5" t="inlineStr">
-        <is>
           <t>Huntsman 癌症研究所·Chandrasekharan 实验室</t>
         </is>
       </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>$7.25</t>
         </is>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>$7.25</t>
-        </is>
-      </c>
-      <c r="H81" s="4" t="inlineStr">
-        <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="I81" s="5" t="inlineStr"/>
+      <c r="H81" s="5" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="n">
@@ -36707,33 +36448,32 @@
           <t>前厅收银员</t>
         </is>
       </c>
-      <c r="C82" s="5" t="inlineStr"/>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>剧场前厅收银、管现金箱、卖零食饮料</t>
+        </is>
+      </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>与他人共同管理餐饮售卖人员和验票志愿者，负责现金箱、库存、迟到观众入场安排、节目单装订与摆放，以及演出前和中场休息期间的…</t>
-        </is>
-      </c>
-      <c r="E82" s="5" t="inlineStr">
-        <is>
           <t>先锋剧院</t>
         </is>
       </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>15-20</t>
+        </is>
+      </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>15-20</t>
+          <t>$11</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>$11</t>
-        </is>
-      </c>
-      <c r="H82" s="4" t="inlineStr">
-        <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="I82" s="5" t="inlineStr">
+      <c r="H82" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -36748,33 +36488,32 @@
           <t>票房售票员</t>
         </is>
       </c>
-      <c r="C83" s="5" t="inlineStr"/>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>售票、换票、收银、答观众问题</t>
+        </is>
+      </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>Pioneer Theatre Company 招聘票房收银员，负责接听电话、售票并回答顾客问题</t>
-        </is>
-      </c>
-      <c r="E83" s="5" t="inlineStr">
-        <is>
           <t>先锋剧院</t>
         </is>
       </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>$10.5</t>
         </is>
       </c>
       <c r="G83" s="4" t="inlineStr">
         <is>
-          <t>$10.5</t>
-        </is>
-      </c>
-      <c r="H83" s="4" t="inlineStr">
-        <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="I83" s="5" t="inlineStr">
+      <c r="H83" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -36789,33 +36528,32 @@
           <t>行政文员</t>
         </is>
       </c>
-      <c r="C84" s="5" t="inlineStr"/>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>处理文件申请、录数据、收发邮件</t>
+        </is>
+      </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>提供常规办公室支持，审核并处理文件和信息申请，维护档案、录入数据并分发邮件</t>
-        </is>
-      </c>
-      <c r="E84" s="5" t="inlineStr">
-        <is>
           <t>校园卡服务</t>
         </is>
       </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>15-19 hours per week</t>
+        </is>
+      </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>15-19 hours per week</t>
+          <t>$15</t>
         </is>
       </c>
       <c r="G84" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="H84" s="4" t="inlineStr">
-        <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="I84" s="5" t="inlineStr">
+      <c r="H84" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -36832,35 +36570,30 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>舞台技术</t>
+          <t>演出后台：挂灯、布线、装卸台、追光灯</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>UtahPresents 是犹他大学的非营利综合艺术演出机构，为校园及周边地区引进舞蹈、音乐会、喜剧、歌剧等项目</t>
-        </is>
-      </c>
-      <c r="E85" s="5" t="inlineStr">
-        <is>
           <t>UtahPresents 演出项目</t>
         </is>
       </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>$16</t>
         </is>
       </c>
       <c r="G85" s="4" t="inlineStr">
         <is>
-          <t>$16</t>
-        </is>
-      </c>
-      <c r="H85" s="4" t="inlineStr">
-        <is>
           <t>2026-11-05</t>
         </is>
       </c>
-      <c r="I85" s="5" t="inlineStr">
+      <c r="H85" s="5" t="inlineStr">
         <is>
           <t>需经验</t>
         </is>
@@ -36875,33 +36608,32 @@
           <t>网球中心前台工作人员</t>
         </is>
       </c>
-      <c r="C86" s="5" t="inlineStr"/>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>收场地费、约场地、接电话、开关场馆</t>
+        </is>
+      </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>为租用室内、室外网球场的顾客收款，办理预约和取消，接听场馆电话并处理顾客的问题，协助场馆经理完成其他前台事务</t>
-        </is>
-      </c>
-      <c r="E86" s="5" t="inlineStr">
-        <is>
           <t>体育部</t>
         </is>
       </c>
+      <c r="E86" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$7.25</t>
         </is>
       </c>
       <c r="G86" s="4" t="inlineStr">
         <is>
-          <t>$7.25</t>
-        </is>
-      </c>
-      <c r="H86" s="4" t="inlineStr">
-        <is>
           <t>2026-11-07</t>
         </is>
       </c>
-      <c r="I86" s="5" t="inlineStr"/>
+      <c r="H86" s="5" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="n">
@@ -36914,35 +36646,30 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>TESOL 教学</t>
+          <t>教 ESL 英语课、备课、记录成绩</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>继续教育与社区参与部门下属的英语语言学院长期招聘线下面授 ESL 兼职教师</t>
-        </is>
-      </c>
-      <c r="E87" s="5" t="inlineStr">
-        <is>
           <t>英语语言学院</t>
         </is>
       </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>$49</t>
         </is>
       </c>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>$49</t>
-        </is>
-      </c>
-      <c r="H87" s="4" t="inlineStr">
-        <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="I87" s="5" t="inlineStr">
+      <c r="H87" s="5" t="inlineStr">
         <is>
           <t>需 TESOL 硕士 + TESOL 证书</t>
         </is>
@@ -36957,33 +36684,32 @@
           <t>住宿招生与外联协调员</t>
         </is>
       </c>
-      <c r="C88" s="5" t="inlineStr"/>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>中心外联招生、摆摊、答咨询</t>
+        </is>
+      </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>犹他大学 Impact &amp; Prosperity Epicenter 是一个以社会影响和共同繁荣为主题的住宿学习社区，通…</t>
-        </is>
-      </c>
-      <c r="E88" s="5" t="inlineStr">
-        <is>
           <t>影响力与繁荣中心</t>
         </is>
       </c>
+      <c r="E88" s="4" t="inlineStr">
+        <is>
+          <t>15-19</t>
+        </is>
+      </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>15-19</t>
+          <t>$12</t>
         </is>
       </c>
       <c r="G88" s="4" t="inlineStr">
         <is>
-          <t>$12</t>
-        </is>
-      </c>
-      <c r="H88" s="4" t="inlineStr">
-        <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="I88" s="5" t="inlineStr"/>
+      <c r="H88" s="5" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="n">
@@ -36996,35 +36722,30 @@
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>摄像</t>
+          <t>舞蹈演出录像和直播</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>在 Marriott Center for Dance 与视听室经理、技术总监、制作总监和舞台经理合作，负责舞蹈学院演出…</t>
-        </is>
-      </c>
-      <c r="E89" s="5" t="inlineStr">
-        <is>
           <t>舞蹈学院</t>
         </is>
       </c>
+      <c r="E89" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>$13.5</t>
         </is>
       </c>
       <c r="G89" s="4" t="inlineStr">
         <is>
-          <t>$13.5</t>
-        </is>
-      </c>
-      <c r="H89" s="4" t="inlineStr">
-        <is>
           <t>2026-12-31</t>
         </is>
       </c>
-      <c r="I89" s="5" t="inlineStr"/>
+      <c r="H89" s="5" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="n">
@@ -37037,41 +36758,36 @@
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>舞台技术</t>
+          <t>舞蹈演出后台：音响、灯光、布景</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>在 Marriott Center for Dance 与制作总监、技术总监、舞台经理和视听室经理合作，为舞蹈学院演出及…</t>
-        </is>
-      </c>
-      <c r="E90" s="5" t="inlineStr">
-        <is>
           <t>舞蹈学院</t>
         </is>
       </c>
+      <c r="E90" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>$13.5</t>
         </is>
       </c>
       <c r="G90" s="4" t="inlineStr">
         <is>
-          <t>$13.5</t>
-        </is>
-      </c>
-      <c r="H90" s="4" t="inlineStr">
-        <is>
           <t>2026-12-31</t>
         </is>
       </c>
-      <c r="I90" s="5" t="inlineStr"/>
+      <c r="H90" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I90"/>
+  <autoFilter ref="A4:H90"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId1"/>

</xml_diff>

<commit_message>
Add experience-equivalency and food-permit notes to README and sheets
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +56,10 @@
     </font>
     <font>
       <color rgb="FFBF8F00"/>
+    </font>
+    <font>
+      <color rgb="00808080"/>
+      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
@@ -99,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -120,7 +124,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -33421,7 +33428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H90"/>
+  <dimension ref="A1:H92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -36783,9 +36790,17 @@
       </c>
       <c r="H90" s="5" t="inlineStr"/>
     </row>
+    <row r="92">
+      <c r="A92" s="10" t="inlineStr">
+        <is>
+          <t>💡 很多写着「需要经验」的岗位，上过两年高等教育（任意专业）通常就能满足（1 年高等教育可折抵 2 年相关工作经验）；有些岗位的语境暗示需要专业对口，需自己判断。食品处理员许可证（Food Handler Permit）很好获得：线上几小时课程 + 少量费用，很多岗位允许入职后再考。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A4:H90"/>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A92:H92"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -36887,7 +36902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -36914,12 +36929,12 @@
     </row>
     <row r="3" ht="6" customHeight="1"/>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>数据概览</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>数值</t>
         </is>
@@ -36978,7 +36993,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>状态图例</t>
         </is>
@@ -37021,7 +37036,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>建议用法</t>
         </is>
@@ -37113,7 +37128,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="inlineStr">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>标签口径</t>
         </is>
@@ -37158,22 +37173,34 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>教育折抵经验</t>
+          <t>需要经验 ≠ 硬门槛</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>仍需结合专业和职位给出的折抵公式判断。</t>
+          <t>很多写着「需要经验」的岗位，上过两年高等教育（任意专业）通常就能满足；有些岗位的语境暗示需要专业对口，需自己判断。</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>食品证</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>食品处理员许可证很好获得：线上几小时课程 + 少量费用，很多岗位允许入职后再考。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>翻译</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>完整中文由 AI 辅助生成；申请前以英文原文为准。</t>
         </is>

</xml_diff>